<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 07:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0BFCC06F-1EC1-48E5-BA70-6C20509150A6}</x14:id>
+          <x14:id>{FF7BCB6E-AF37-43A4-9B9A-8A741014FEB5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DAD676A9-C01D-4B5B-90D0-6A8B06FA6D0D}</x14:id>
+          <x14:id>{AD40467A-9316-49B1-BB87-FA85B6F45116}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6195957B-6BD3-46A2-9FBA-D09FD3D20A19}</x14:id>
+          <x14:id>{D577F12B-B72A-462D-9F79-446110D07171}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{15B5603E-8678-4594-870C-C972591626DC}</x14:id>
+          <x14:id>{414873CE-C0AE-4C5D-8580-F5ABFADAA8E2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0BFCC06F-1EC1-48E5-BA70-6C20509150A6}">
+          <x14:cfRule type="dataBar" id="{FF7BCB6E-AF37-43A4-9B9A-8A741014FEB5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DAD676A9-C01D-4B5B-90D0-6A8B06FA6D0D}">
+          <x14:cfRule type="dataBar" id="{AD40467A-9316-49B1-BB87-FA85B6F45116}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6195957B-6BD3-46A2-9FBA-D09FD3D20A19}">
+          <x14:cfRule type="dataBar" id="{D577F12B-B72A-462D-9F79-446110D07171}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{15B5603E-8678-4594-870C-C972591626DC}">
+          <x14:cfRule type="dataBar" id="{414873CE-C0AE-4C5D-8580-F5ABFADAA8E2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2A797029-00D2-4F7A-A8CC-A11033102761}</x14:id>
+          <x14:id>{06994663-BCA6-4C14-8698-6EAD2A2A005B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E406DAA2-DA2D-4EBD-B39B-67F6432C7037}</x14:id>
+          <x14:id>{8497CC21-0F87-4C4E-9B87-766BEE67A076}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F390352A-925E-4FFE-B900-F7B737A7F260}</x14:id>
+          <x14:id>{DDCE8314-70F2-48E9-86BB-B49C301C7310}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8C5E896D-2CEC-45D5-865E-71D11041860C}</x14:id>
+          <x14:id>{D0548956-6AC4-49C7-A513-052E964C06BC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2A797029-00D2-4F7A-A8CC-A11033102761}">
+          <x14:cfRule type="dataBar" id="{06994663-BCA6-4C14-8698-6EAD2A2A005B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E406DAA2-DA2D-4EBD-B39B-67F6432C7037}">
+          <x14:cfRule type="dataBar" id="{8497CC21-0F87-4C4E-9B87-766BEE67A076}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F390352A-925E-4FFE-B900-F7B737A7F260}">
+          <x14:cfRule type="dataBar" id="{DDCE8314-70F2-48E9-86BB-B49C301C7310}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8C5E896D-2CEC-45D5-865E-71D11041860C}">
+          <x14:cfRule type="dataBar" id="{D0548956-6AC4-49C7-A513-052E964C06BC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FF7BCB6E-AF37-43A4-9B9A-8A741014FEB5}</x14:id>
+          <x14:id>{7C749BD8-5324-495F-A0F0-DF88E3BF9A43}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AD40467A-9316-49B1-BB87-FA85B6F45116}</x14:id>
+          <x14:id>{6ECB13B8-1D88-4946-A98F-700DDE6E1C77}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D577F12B-B72A-462D-9F79-446110D07171}</x14:id>
+          <x14:id>{9C17C229-A59C-467D-AFA3-329AAAEA880B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{414873CE-C0AE-4C5D-8580-F5ABFADAA8E2}</x14:id>
+          <x14:id>{2A8F4A9D-2EBA-40A8-B1B1-847334344E04}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FF7BCB6E-AF37-43A4-9B9A-8A741014FEB5}">
+          <x14:cfRule type="dataBar" id="{7C749BD8-5324-495F-A0F0-DF88E3BF9A43}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AD40467A-9316-49B1-BB87-FA85B6F45116}">
+          <x14:cfRule type="dataBar" id="{6ECB13B8-1D88-4946-A98F-700DDE6E1C77}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D577F12B-B72A-462D-9F79-446110D07171}">
+          <x14:cfRule type="dataBar" id="{9C17C229-A59C-467D-AFA3-329AAAEA880B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{414873CE-C0AE-4C5D-8580-F5ABFADAA8E2}">
+          <x14:cfRule type="dataBar" id="{2A8F4A9D-2EBA-40A8-B1B1-847334344E04}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{06994663-BCA6-4C14-8698-6EAD2A2A005B}</x14:id>
+          <x14:id>{473D00FB-B881-4FD3-BC1F-26C06ED7D661}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8497CC21-0F87-4C4E-9B87-766BEE67A076}</x14:id>
+          <x14:id>{31BEB778-883E-436A-9FE9-9981D855EBDE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DDCE8314-70F2-48E9-86BB-B49C301C7310}</x14:id>
+          <x14:id>{5D1A972B-8392-4877-84C3-C5C1CC3B4CBA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D0548956-6AC4-49C7-A513-052E964C06BC}</x14:id>
+          <x14:id>{59B10002-5593-47F0-A856-8BEEF9A289CA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{06994663-BCA6-4C14-8698-6EAD2A2A005B}">
+          <x14:cfRule type="dataBar" id="{473D00FB-B881-4FD3-BC1F-26C06ED7D661}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8497CC21-0F87-4C4E-9B87-766BEE67A076}">
+          <x14:cfRule type="dataBar" id="{31BEB778-883E-436A-9FE9-9981D855EBDE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DDCE8314-70F2-48E9-86BB-B49C301C7310}">
+          <x14:cfRule type="dataBar" id="{5D1A972B-8392-4877-84C3-C5C1CC3B4CBA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D0548956-6AC4-49C7-A513-052E964C06BC}">
+          <x14:cfRule type="dataBar" id="{59B10002-5593-47F0-A856-8BEEF9A289CA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7C749BD8-5324-495F-A0F0-DF88E3BF9A43}</x14:id>
+          <x14:id>{3ECC9189-6E1B-4D13-8CED-2C42259EA955}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6ECB13B8-1D88-4946-A98F-700DDE6E1C77}</x14:id>
+          <x14:id>{E8374693-7CE0-4F60-A407-F42331610A09}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9C17C229-A59C-467D-AFA3-329AAAEA880B}</x14:id>
+          <x14:id>{EE1ED37A-8583-4B8A-BE89-7E80BC08C209}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2A8F4A9D-2EBA-40A8-B1B1-847334344E04}</x14:id>
+          <x14:id>{E0AE44D1-8029-435E-B5E8-530699D1C8AE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7C749BD8-5324-495F-A0F0-DF88E3BF9A43}">
+          <x14:cfRule type="dataBar" id="{3ECC9189-6E1B-4D13-8CED-2C42259EA955}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6ECB13B8-1D88-4946-A98F-700DDE6E1C77}">
+          <x14:cfRule type="dataBar" id="{E8374693-7CE0-4F60-A407-F42331610A09}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9C17C229-A59C-467D-AFA3-329AAAEA880B}">
+          <x14:cfRule type="dataBar" id="{EE1ED37A-8583-4B8A-BE89-7E80BC08C209}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2A8F4A9D-2EBA-40A8-B1B1-847334344E04}">
+          <x14:cfRule type="dataBar" id="{E0AE44D1-8029-435E-B5E8-530699D1C8AE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{473D00FB-B881-4FD3-BC1F-26C06ED7D661}</x14:id>
+          <x14:id>{42AE71D9-5CD6-4E4E-872E-4CF62CA311FC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{31BEB778-883E-436A-9FE9-9981D855EBDE}</x14:id>
+          <x14:id>{1C78F0F0-7012-41E2-9CD5-D388566513C8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5D1A972B-8392-4877-84C3-C5C1CC3B4CBA}</x14:id>
+          <x14:id>{D61AE91C-EB6D-40F0-B586-5833015DAF39}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{59B10002-5593-47F0-A856-8BEEF9A289CA}</x14:id>
+          <x14:id>{F0BD4821-8D37-4765-80C1-C1AAC288B0F6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{473D00FB-B881-4FD3-BC1F-26C06ED7D661}">
+          <x14:cfRule type="dataBar" id="{42AE71D9-5CD6-4E4E-872E-4CF62CA311FC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{31BEB778-883E-436A-9FE9-9981D855EBDE}">
+          <x14:cfRule type="dataBar" id="{1C78F0F0-7012-41E2-9CD5-D388566513C8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5D1A972B-8392-4877-84C3-C5C1CC3B4CBA}">
+          <x14:cfRule type="dataBar" id="{D61AE91C-EB6D-40F0-B586-5833015DAF39}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{59B10002-5593-47F0-A856-8BEEF9A289CA}">
+          <x14:cfRule type="dataBar" id="{F0BD4821-8D37-4765-80C1-C1AAC288B0F6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3ECC9189-6E1B-4D13-8CED-2C42259EA955}</x14:id>
+          <x14:id>{59BB2A40-D379-4BD2-8CB1-44DFE557A6E5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E8374693-7CE0-4F60-A407-F42331610A09}</x14:id>
+          <x14:id>{709040CC-BF97-4FCC-86D4-198B23F19DA3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EE1ED37A-8583-4B8A-BE89-7E80BC08C209}</x14:id>
+          <x14:id>{F0A2CA0F-17CE-4A1B-A619-B30C07376DB4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E0AE44D1-8029-435E-B5E8-530699D1C8AE}</x14:id>
+          <x14:id>{E2EC64BF-625F-4625-AE4E-A1E0D5450D2E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3ECC9189-6E1B-4D13-8CED-2C42259EA955}">
+          <x14:cfRule type="dataBar" id="{59BB2A40-D379-4BD2-8CB1-44DFE557A6E5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E8374693-7CE0-4F60-A407-F42331610A09}">
+          <x14:cfRule type="dataBar" id="{709040CC-BF97-4FCC-86D4-198B23F19DA3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EE1ED37A-8583-4B8A-BE89-7E80BC08C209}">
+          <x14:cfRule type="dataBar" id="{F0A2CA0F-17CE-4A1B-A619-B30C07376DB4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E0AE44D1-8029-435E-B5E8-530699D1C8AE}">
+          <x14:cfRule type="dataBar" id="{E2EC64BF-625F-4625-AE4E-A1E0D5450D2E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{42AE71D9-5CD6-4E4E-872E-4CF62CA311FC}</x14:id>
+          <x14:id>{5EDE94DE-FB9D-43F0-942D-EF57DEDBFDA0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1C78F0F0-7012-41E2-9CD5-D388566513C8}</x14:id>
+          <x14:id>{3F24809D-03BF-4BF7-9558-B53686DB91E1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D61AE91C-EB6D-40F0-B586-5833015DAF39}</x14:id>
+          <x14:id>{340CC9C7-7AB1-4881-8803-AC64EF64981E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F0BD4821-8D37-4765-80C1-C1AAC288B0F6}</x14:id>
+          <x14:id>{C66E7CB4-E8D2-42F7-BD44-B578E4D125BC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{42AE71D9-5CD6-4E4E-872E-4CF62CA311FC}">
+          <x14:cfRule type="dataBar" id="{5EDE94DE-FB9D-43F0-942D-EF57DEDBFDA0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1C78F0F0-7012-41E2-9CD5-D388566513C8}">
+          <x14:cfRule type="dataBar" id="{3F24809D-03BF-4BF7-9558-B53686DB91E1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D61AE91C-EB6D-40F0-B586-5833015DAF39}">
+          <x14:cfRule type="dataBar" id="{340CC9C7-7AB1-4881-8803-AC64EF64981E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F0BD4821-8D37-4765-80C1-C1AAC288B0F6}">
+          <x14:cfRule type="dataBar" id="{C66E7CB4-E8D2-42F7-BD44-B578E4D125BC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{59BB2A40-D379-4BD2-8CB1-44DFE557A6E5}</x14:id>
+          <x14:id>{4F72A895-7A34-4690-90F1-5C63A66A9988}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{709040CC-BF97-4FCC-86D4-198B23F19DA3}</x14:id>
+          <x14:id>{1E9AD4D7-46CF-4ECA-A44E-F30F1679B2EA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F0A2CA0F-17CE-4A1B-A619-B30C07376DB4}</x14:id>
+          <x14:id>{0719A0C9-F947-49FC-90D8-09BEF1303368}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E2EC64BF-625F-4625-AE4E-A1E0D5450D2E}</x14:id>
+          <x14:id>{A13FB91A-4DA8-4996-9B67-34650EEEF04D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{59BB2A40-D379-4BD2-8CB1-44DFE557A6E5}">
+          <x14:cfRule type="dataBar" id="{4F72A895-7A34-4690-90F1-5C63A66A9988}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{709040CC-BF97-4FCC-86D4-198B23F19DA3}">
+          <x14:cfRule type="dataBar" id="{1E9AD4D7-46CF-4ECA-A44E-F30F1679B2EA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F0A2CA0F-17CE-4A1B-A619-B30C07376DB4}">
+          <x14:cfRule type="dataBar" id="{0719A0C9-F947-49FC-90D8-09BEF1303368}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E2EC64BF-625F-4625-AE4E-A1E0D5450D2E}">
+          <x14:cfRule type="dataBar" id="{A13FB91A-4DA8-4996-9B67-34650EEEF04D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5EDE94DE-FB9D-43F0-942D-EF57DEDBFDA0}</x14:id>
+          <x14:id>{4F7DAFDC-ACC2-4B23-BC4A-AB28D6E9FF4D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3F24809D-03BF-4BF7-9558-B53686DB91E1}</x14:id>
+          <x14:id>{C132ECCA-C616-4418-BA7D-70D8F5F29016}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{340CC9C7-7AB1-4881-8803-AC64EF64981E}</x14:id>
+          <x14:id>{CAACC8F5-6D4B-4106-B68A-86D0132A1879}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C66E7CB4-E8D2-42F7-BD44-B578E4D125BC}</x14:id>
+          <x14:id>{3E14EA23-9949-406A-8C0F-6EB41B3788A0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5EDE94DE-FB9D-43F0-942D-EF57DEDBFDA0}">
+          <x14:cfRule type="dataBar" id="{4F7DAFDC-ACC2-4B23-BC4A-AB28D6E9FF4D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3F24809D-03BF-4BF7-9558-B53686DB91E1}">
+          <x14:cfRule type="dataBar" id="{C132ECCA-C616-4418-BA7D-70D8F5F29016}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{340CC9C7-7AB1-4881-8803-AC64EF64981E}">
+          <x14:cfRule type="dataBar" id="{CAACC8F5-6D4B-4106-B68A-86D0132A1879}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C66E7CB4-E8D2-42F7-BD44-B578E4D125BC}">
+          <x14:cfRule type="dataBar" id="{3E14EA23-9949-406A-8C0F-6EB41B3788A0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4F72A895-7A34-4690-90F1-5C63A66A9988}</x14:id>
+          <x14:id>{8DA65D8B-3769-46B6-8BDA-2EDCDAC62643}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1E9AD4D7-46CF-4ECA-A44E-F30F1679B2EA}</x14:id>
+          <x14:id>{EC2FEBD5-9C64-4F54-8BE7-25DAE218CB29}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0719A0C9-F947-49FC-90D8-09BEF1303368}</x14:id>
+          <x14:id>{22E0206D-DA42-4F73-81BA-77D8DB84E8A8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A13FB91A-4DA8-4996-9B67-34650EEEF04D}</x14:id>
+          <x14:id>{74D12373-1FD4-46FB-8763-AC48F1526CF0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4F72A895-7A34-4690-90F1-5C63A66A9988}">
+          <x14:cfRule type="dataBar" id="{8DA65D8B-3769-46B6-8BDA-2EDCDAC62643}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1E9AD4D7-46CF-4ECA-A44E-F30F1679B2EA}">
+          <x14:cfRule type="dataBar" id="{EC2FEBD5-9C64-4F54-8BE7-25DAE218CB29}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0719A0C9-F947-49FC-90D8-09BEF1303368}">
+          <x14:cfRule type="dataBar" id="{22E0206D-DA42-4F73-81BA-77D8DB84E8A8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A13FB91A-4DA8-4996-9B67-34650EEEF04D}">
+          <x14:cfRule type="dataBar" id="{74D12373-1FD4-46FB-8763-AC48F1526CF0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4F7DAFDC-ACC2-4B23-BC4A-AB28D6E9FF4D}</x14:id>
+          <x14:id>{6879AA91-F5A8-4D4D-B20E-3E8092832276}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C132ECCA-C616-4418-BA7D-70D8F5F29016}</x14:id>
+          <x14:id>{8303DD46-8624-4F2C-B0AC-939934D1D780}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CAACC8F5-6D4B-4106-B68A-86D0132A1879}</x14:id>
+          <x14:id>{C6EAB8F7-0736-4854-AF94-279A41684D95}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3E14EA23-9949-406A-8C0F-6EB41B3788A0}</x14:id>
+          <x14:id>{B10B9EA5-76E8-49BD-BC76-C2CDDF4BC0AF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4F7DAFDC-ACC2-4B23-BC4A-AB28D6E9FF4D}">
+          <x14:cfRule type="dataBar" id="{6879AA91-F5A8-4D4D-B20E-3E8092832276}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C132ECCA-C616-4418-BA7D-70D8F5F29016}">
+          <x14:cfRule type="dataBar" id="{8303DD46-8624-4F2C-B0AC-939934D1D780}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CAACC8F5-6D4B-4106-B68A-86D0132A1879}">
+          <x14:cfRule type="dataBar" id="{C6EAB8F7-0736-4854-AF94-279A41684D95}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3E14EA23-9949-406A-8C0F-6EB41B3788A0}">
+          <x14:cfRule type="dataBar" id="{B10B9EA5-76E8-49BD-BC76-C2CDDF4BC0AF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8DA65D8B-3769-46B6-8BDA-2EDCDAC62643}</x14:id>
+          <x14:id>{2A0F28FE-53AF-46B2-AAB3-7F3557273990}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EC2FEBD5-9C64-4F54-8BE7-25DAE218CB29}</x14:id>
+          <x14:id>{020D44CF-6BA8-4FF3-B6B6-47B7E3179E48}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{22E0206D-DA42-4F73-81BA-77D8DB84E8A8}</x14:id>
+          <x14:id>{CD2E42D6-C2E9-4591-9102-58CC065794C0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{74D12373-1FD4-46FB-8763-AC48F1526CF0}</x14:id>
+          <x14:id>{6CECB11D-732B-430D-82DF-2866658CABE9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8DA65D8B-3769-46B6-8BDA-2EDCDAC62643}">
+          <x14:cfRule type="dataBar" id="{2A0F28FE-53AF-46B2-AAB3-7F3557273990}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EC2FEBD5-9C64-4F54-8BE7-25DAE218CB29}">
+          <x14:cfRule type="dataBar" id="{020D44CF-6BA8-4FF3-B6B6-47B7E3179E48}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{22E0206D-DA42-4F73-81BA-77D8DB84E8A8}">
+          <x14:cfRule type="dataBar" id="{CD2E42D6-C2E9-4591-9102-58CC065794C0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{74D12373-1FD4-46FB-8763-AC48F1526CF0}">
+          <x14:cfRule type="dataBar" id="{6CECB11D-732B-430D-82DF-2866658CABE9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6879AA91-F5A8-4D4D-B20E-3E8092832276}</x14:id>
+          <x14:id>{E26787E9-8EC8-465E-8FF1-649A8180EA0C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8303DD46-8624-4F2C-B0AC-939934D1D780}</x14:id>
+          <x14:id>{CEB09826-8A31-4145-9BB3-267D9677F522}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C6EAB8F7-0736-4854-AF94-279A41684D95}</x14:id>
+          <x14:id>{94CAD790-6499-468B-8ADE-79F5966DA5A1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B10B9EA5-76E8-49BD-BC76-C2CDDF4BC0AF}</x14:id>
+          <x14:id>{3D309DFB-F8A6-47EF-94ED-A73D2BFE6077}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6879AA91-F5A8-4D4D-B20E-3E8092832276}">
+          <x14:cfRule type="dataBar" id="{E26787E9-8EC8-465E-8FF1-649A8180EA0C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8303DD46-8624-4F2C-B0AC-939934D1D780}">
+          <x14:cfRule type="dataBar" id="{CEB09826-8A31-4145-9BB3-267D9677F522}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C6EAB8F7-0736-4854-AF94-279A41684D95}">
+          <x14:cfRule type="dataBar" id="{94CAD790-6499-468B-8ADE-79F5966DA5A1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B10B9EA5-76E8-49BD-BC76-C2CDDF4BC0AF}">
+          <x14:cfRule type="dataBar" id="{3D309DFB-F8A6-47EF-94ED-A73D2BFE6077}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2A0F28FE-53AF-46B2-AAB3-7F3557273990}</x14:id>
+          <x14:id>{E2E117A9-9264-439D-95EB-9452761636B7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{020D44CF-6BA8-4FF3-B6B6-47B7E3179E48}</x14:id>
+          <x14:id>{0FA72F70-0B30-4810-9463-E238602484CD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CD2E42D6-C2E9-4591-9102-58CC065794C0}</x14:id>
+          <x14:id>{BC56ED6A-C999-4CDB-97F7-9C71D2CCB7D5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6CECB11D-732B-430D-82DF-2866658CABE9}</x14:id>
+          <x14:id>{30D0FEB6-828F-47EA-A0C9-1A8EBBB527B0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2A0F28FE-53AF-46B2-AAB3-7F3557273990}">
+          <x14:cfRule type="dataBar" id="{E2E117A9-9264-439D-95EB-9452761636B7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{020D44CF-6BA8-4FF3-B6B6-47B7E3179E48}">
+          <x14:cfRule type="dataBar" id="{0FA72F70-0B30-4810-9463-E238602484CD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CD2E42D6-C2E9-4591-9102-58CC065794C0}">
+          <x14:cfRule type="dataBar" id="{BC56ED6A-C999-4CDB-97F7-9C71D2CCB7D5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6CECB11D-732B-430D-82DF-2866658CABE9}">
+          <x14:cfRule type="dataBar" id="{30D0FEB6-828F-47EA-A0C9-1A8EBBB527B0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E26787E9-8EC8-465E-8FF1-649A8180EA0C}</x14:id>
+          <x14:id>{CF5A3C31-8B5B-4147-AACB-A73591FEA436}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CEB09826-8A31-4145-9BB3-267D9677F522}</x14:id>
+          <x14:id>{67AEE36A-B95B-46EB-AA30-AF9D6FE7A15A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{94CAD790-6499-468B-8ADE-79F5966DA5A1}</x14:id>
+          <x14:id>{E00B8B37-B85D-442F-B1DC-7E6F7596208B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3D309DFB-F8A6-47EF-94ED-A73D2BFE6077}</x14:id>
+          <x14:id>{7E9DF770-238C-4FA1-8D04-2EEC2011439E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E26787E9-8EC8-465E-8FF1-649A8180EA0C}">
+          <x14:cfRule type="dataBar" id="{CF5A3C31-8B5B-4147-AACB-A73591FEA436}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CEB09826-8A31-4145-9BB3-267D9677F522}">
+          <x14:cfRule type="dataBar" id="{67AEE36A-B95B-46EB-AA30-AF9D6FE7A15A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{94CAD790-6499-468B-8ADE-79F5966DA5A1}">
+          <x14:cfRule type="dataBar" id="{E00B8B37-B85D-442F-B1DC-7E6F7596208B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3D309DFB-F8A6-47EF-94ED-A73D2BFE6077}">
+          <x14:cfRule type="dataBar" id="{7E9DF770-238C-4FA1-8D04-2EEC2011439E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E2E117A9-9264-439D-95EB-9452761636B7}</x14:id>
+          <x14:id>{1AAA2E39-E29B-416C-9F1A-4A55214FFDAD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0FA72F70-0B30-4810-9463-E238602484CD}</x14:id>
+          <x14:id>{DB8B8DAA-A4D9-4734-AA85-C3A5C609C6D2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BC56ED6A-C999-4CDB-97F7-9C71D2CCB7D5}</x14:id>
+          <x14:id>{F313BA1F-D781-44D7-A330-6B8337EBE32C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{30D0FEB6-828F-47EA-A0C9-1A8EBBB527B0}</x14:id>
+          <x14:id>{9403E5F9-2F2B-4459-8FB3-E0CFAE736D9F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E2E117A9-9264-439D-95EB-9452761636B7}">
+          <x14:cfRule type="dataBar" id="{1AAA2E39-E29B-416C-9F1A-4A55214FFDAD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0FA72F70-0B30-4810-9463-E238602484CD}">
+          <x14:cfRule type="dataBar" id="{DB8B8DAA-A4D9-4734-AA85-C3A5C609C6D2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BC56ED6A-C999-4CDB-97F7-9C71D2CCB7D5}">
+          <x14:cfRule type="dataBar" id="{F313BA1F-D781-44D7-A330-6B8337EBE32C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{30D0FEB6-828F-47EA-A0C9-1A8EBBB527B0}">
+          <x14:cfRule type="dataBar" id="{9403E5F9-2F2B-4459-8FB3-E0CFAE736D9F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CF5A3C31-8B5B-4147-AACB-A73591FEA436}</x14:id>
+          <x14:id>{C42964A4-A412-4F1E-ACD3-198B6929C514}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{67AEE36A-B95B-46EB-AA30-AF9D6FE7A15A}</x14:id>
+          <x14:id>{0D276975-5283-42B6-B50C-740FE513CD8A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E00B8B37-B85D-442F-B1DC-7E6F7596208B}</x14:id>
+          <x14:id>{08A2B13E-A87D-4B38-935F-99EB2C46CDC6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7E9DF770-238C-4FA1-8D04-2EEC2011439E}</x14:id>
+          <x14:id>{AF118DF6-3D86-45F8-9403-BD109CD041ED}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CF5A3C31-8B5B-4147-AACB-A73591FEA436}">
+          <x14:cfRule type="dataBar" id="{C42964A4-A412-4F1E-ACD3-198B6929C514}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{67AEE36A-B95B-46EB-AA30-AF9D6FE7A15A}">
+          <x14:cfRule type="dataBar" id="{0D276975-5283-42B6-B50C-740FE513CD8A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E00B8B37-B85D-442F-B1DC-7E6F7596208B}">
+          <x14:cfRule type="dataBar" id="{08A2B13E-A87D-4B38-935F-99EB2C46CDC6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7E9DF770-238C-4FA1-8D04-2EEC2011439E}">
+          <x14:cfRule type="dataBar" id="{AF118DF6-3D86-45F8-9403-BD109CD041ED}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1AAA2E39-E29B-416C-9F1A-4A55214FFDAD}</x14:id>
+          <x14:id>{BFDD972F-169B-4E24-907B-60839456497E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DB8B8DAA-A4D9-4734-AA85-C3A5C609C6D2}</x14:id>
+          <x14:id>{D12D062E-3C35-494C-BD00-AEF2B58B7E6D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F313BA1F-D781-44D7-A330-6B8337EBE32C}</x14:id>
+          <x14:id>{D06978B3-2E54-418D-8C60-2F1A85CDABD6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9403E5F9-2F2B-4459-8FB3-E0CFAE736D9F}</x14:id>
+          <x14:id>{53FE7F91-A2F8-4C92-82D5-07B48FD694C1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1AAA2E39-E29B-416C-9F1A-4A55214FFDAD}">
+          <x14:cfRule type="dataBar" id="{BFDD972F-169B-4E24-907B-60839456497E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DB8B8DAA-A4D9-4734-AA85-C3A5C609C6D2}">
+          <x14:cfRule type="dataBar" id="{D12D062E-3C35-494C-BD00-AEF2B58B7E6D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F313BA1F-D781-44D7-A330-6B8337EBE32C}">
+          <x14:cfRule type="dataBar" id="{D06978B3-2E54-418D-8C60-2F1A85CDABD6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9403E5F9-2F2B-4459-8FB3-E0CFAE736D9F}">
+          <x14:cfRule type="dataBar" id="{53FE7F91-A2F8-4C92-82D5-07B48FD694C1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C42964A4-A412-4F1E-ACD3-198B6929C514}</x14:id>
+          <x14:id>{5A17E393-1027-4AEF-B7D3-5798967A6958}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0D276975-5283-42B6-B50C-740FE513CD8A}</x14:id>
+          <x14:id>{B88895F9-4AB2-4AF6-BF58-005DD15D2A9B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{08A2B13E-A87D-4B38-935F-99EB2C46CDC6}</x14:id>
+          <x14:id>{998D07F3-1AD6-4EE1-BF2B-D725EBBC9A71}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AF118DF6-3D86-45F8-9403-BD109CD041ED}</x14:id>
+          <x14:id>{E54BEBFD-9690-4DA0-B8E2-E7CC0A1C56FA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C42964A4-A412-4F1E-ACD3-198B6929C514}">
+          <x14:cfRule type="dataBar" id="{5A17E393-1027-4AEF-B7D3-5798967A6958}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0D276975-5283-42B6-B50C-740FE513CD8A}">
+          <x14:cfRule type="dataBar" id="{B88895F9-4AB2-4AF6-BF58-005DD15D2A9B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{08A2B13E-A87D-4B38-935F-99EB2C46CDC6}">
+          <x14:cfRule type="dataBar" id="{998D07F3-1AD6-4EE1-BF2B-D725EBBC9A71}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AF118DF6-3D86-45F8-9403-BD109CD041ED}">
+          <x14:cfRule type="dataBar" id="{E54BEBFD-9690-4DA0-B8E2-E7CC0A1C56FA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BFDD972F-169B-4E24-907B-60839456497E}</x14:id>
+          <x14:id>{77700F2F-AA79-48C6-BDF6-0F50821AFE98}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D12D062E-3C35-494C-BD00-AEF2B58B7E6D}</x14:id>
+          <x14:id>{C57783CA-DA1A-4D4F-BC5B-888C2A3EAB93}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D06978B3-2E54-418D-8C60-2F1A85CDABD6}</x14:id>
+          <x14:id>{63F17E22-7407-4F8C-8645-CA0B47713399}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{53FE7F91-A2F8-4C92-82D5-07B48FD694C1}</x14:id>
+          <x14:id>{1D186B90-B19D-4072-809B-076DAAE7E66A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BFDD972F-169B-4E24-907B-60839456497E}">
+          <x14:cfRule type="dataBar" id="{77700F2F-AA79-48C6-BDF6-0F50821AFE98}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D12D062E-3C35-494C-BD00-AEF2B58B7E6D}">
+          <x14:cfRule type="dataBar" id="{C57783CA-DA1A-4D4F-BC5B-888C2A3EAB93}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D06978B3-2E54-418D-8C60-2F1A85CDABD6}">
+          <x14:cfRule type="dataBar" id="{63F17E22-7407-4F8C-8645-CA0B47713399}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{53FE7F91-A2F8-4C92-82D5-07B48FD694C1}">
+          <x14:cfRule type="dataBar" id="{1D186B90-B19D-4072-809B-076DAAE7E66A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5A17E393-1027-4AEF-B7D3-5798967A6958}</x14:id>
+          <x14:id>{1A9952DF-CF59-42D6-9DF7-B761436152A6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B88895F9-4AB2-4AF6-BF58-005DD15D2A9B}</x14:id>
+          <x14:id>{996ED2F8-0A21-41B3-82EA-1CC25EDE355B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{998D07F3-1AD6-4EE1-BF2B-D725EBBC9A71}</x14:id>
+          <x14:id>{AA2C27C9-71BF-47EF-8FDA-54EBAED026CB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E54BEBFD-9690-4DA0-B8E2-E7CC0A1C56FA}</x14:id>
+          <x14:id>{02D7B180-7122-42DE-A525-FFC9328D6462}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5A17E393-1027-4AEF-B7D3-5798967A6958}">
+          <x14:cfRule type="dataBar" id="{1A9952DF-CF59-42D6-9DF7-B761436152A6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B88895F9-4AB2-4AF6-BF58-005DD15D2A9B}">
+          <x14:cfRule type="dataBar" id="{996ED2F8-0A21-41B3-82EA-1CC25EDE355B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{998D07F3-1AD6-4EE1-BF2B-D725EBBC9A71}">
+          <x14:cfRule type="dataBar" id="{AA2C27C9-71BF-47EF-8FDA-54EBAED026CB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E54BEBFD-9690-4DA0-B8E2-E7CC0A1C56FA}">
+          <x14:cfRule type="dataBar" id="{02D7B180-7122-42DE-A525-FFC9328D6462}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{77700F2F-AA79-48C6-BDF6-0F50821AFE98}</x14:id>
+          <x14:id>{3C100F65-F45C-4EF9-82EA-D1D08D43C65D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C57783CA-DA1A-4D4F-BC5B-888C2A3EAB93}</x14:id>
+          <x14:id>{0EDE7E4B-F633-4B39-B910-D1746CE401CC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{63F17E22-7407-4F8C-8645-CA0B47713399}</x14:id>
+          <x14:id>{2D7C04E1-42E1-4D3B-A233-4E91EC8CE039}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1D186B90-B19D-4072-809B-076DAAE7E66A}</x14:id>
+          <x14:id>{F2B4DCE3-35D6-4EEF-86EC-00330BBDE883}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{77700F2F-AA79-48C6-BDF6-0F50821AFE98}">
+          <x14:cfRule type="dataBar" id="{3C100F65-F45C-4EF9-82EA-D1D08D43C65D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C57783CA-DA1A-4D4F-BC5B-888C2A3EAB93}">
+          <x14:cfRule type="dataBar" id="{0EDE7E4B-F633-4B39-B910-D1746CE401CC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{63F17E22-7407-4F8C-8645-CA0B47713399}">
+          <x14:cfRule type="dataBar" id="{2D7C04E1-42E1-4D3B-A233-4E91EC8CE039}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1D186B90-B19D-4072-809B-076DAAE7E66A}">
+          <x14:cfRule type="dataBar" id="{F2B4DCE3-35D6-4EEF-86EC-00330BBDE883}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1A9952DF-CF59-42D6-9DF7-B761436152A6}</x14:id>
+          <x14:id>{423AE9B3-9F64-4DE8-93B1-6E876014A683}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{996ED2F8-0A21-41B3-82EA-1CC25EDE355B}</x14:id>
+          <x14:id>{2DBDE1C9-45A7-497C-8DD2-937F05618E89}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AA2C27C9-71BF-47EF-8FDA-54EBAED026CB}</x14:id>
+          <x14:id>{24DD04D6-E1F2-4C8E-B559-A60E7F3FCBBF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{02D7B180-7122-42DE-A525-FFC9328D6462}</x14:id>
+          <x14:id>{3A5911B4-42E6-4950-BBEA-5329448F88C7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1A9952DF-CF59-42D6-9DF7-B761436152A6}">
+          <x14:cfRule type="dataBar" id="{423AE9B3-9F64-4DE8-93B1-6E876014A683}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{996ED2F8-0A21-41B3-82EA-1CC25EDE355B}">
+          <x14:cfRule type="dataBar" id="{2DBDE1C9-45A7-497C-8DD2-937F05618E89}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AA2C27C9-71BF-47EF-8FDA-54EBAED026CB}">
+          <x14:cfRule type="dataBar" id="{24DD04D6-E1F2-4C8E-B559-A60E7F3FCBBF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{02D7B180-7122-42DE-A525-FFC9328D6462}">
+          <x14:cfRule type="dataBar" id="{3A5911B4-42E6-4950-BBEA-5329448F88C7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 08:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3C100F65-F45C-4EF9-82EA-D1D08D43C65D}</x14:id>
+          <x14:id>{98E7BD88-188A-460A-9BB9-C15A4B7456EA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0EDE7E4B-F633-4B39-B910-D1746CE401CC}</x14:id>
+          <x14:id>{70DC13FA-3455-4DFA-9EC5-59D56846EB68}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2D7C04E1-42E1-4D3B-A233-4E91EC8CE039}</x14:id>
+          <x14:id>{62DD2A53-1661-4128-BCB8-73284A9CC0FB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F2B4DCE3-35D6-4EEF-86EC-00330BBDE883}</x14:id>
+          <x14:id>{87470643-D778-4DD7-A43F-0F9AA20F3131}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3C100F65-F45C-4EF9-82EA-D1D08D43C65D}">
+          <x14:cfRule type="dataBar" id="{98E7BD88-188A-460A-9BB9-C15A4B7456EA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0EDE7E4B-F633-4B39-B910-D1746CE401CC}">
+          <x14:cfRule type="dataBar" id="{70DC13FA-3455-4DFA-9EC5-59D56846EB68}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2D7C04E1-42E1-4D3B-A233-4E91EC8CE039}">
+          <x14:cfRule type="dataBar" id="{62DD2A53-1661-4128-BCB8-73284A9CC0FB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F2B4DCE3-35D6-4EEF-86EC-00330BBDE883}">
+          <x14:cfRule type="dataBar" id="{87470643-D778-4DD7-A43F-0F9AA20F3131}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{423AE9B3-9F64-4DE8-93B1-6E876014A683}</x14:id>
+          <x14:id>{5250E87C-DB5F-49E7-9FAD-E5B100C9A403}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2DBDE1C9-45A7-497C-8DD2-937F05618E89}</x14:id>
+          <x14:id>{C39CBEF7-CCA3-4D5C-8D1D-302310DB5396}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{24DD04D6-E1F2-4C8E-B559-A60E7F3FCBBF}</x14:id>
+          <x14:id>{63A4C655-CD3E-483D-90B2-DE0665E8E510}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3A5911B4-42E6-4950-BBEA-5329448F88C7}</x14:id>
+          <x14:id>{D190B475-D8BD-4962-B6A5-413616CFB2B1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{423AE9B3-9F64-4DE8-93B1-6E876014A683}">
+          <x14:cfRule type="dataBar" id="{5250E87C-DB5F-49E7-9FAD-E5B100C9A403}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2DBDE1C9-45A7-497C-8DD2-937F05618E89}">
+          <x14:cfRule type="dataBar" id="{C39CBEF7-CCA3-4D5C-8D1D-302310DB5396}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{24DD04D6-E1F2-4C8E-B559-A60E7F3FCBBF}">
+          <x14:cfRule type="dataBar" id="{63A4C655-CD3E-483D-90B2-DE0665E8E510}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3A5911B4-42E6-4950-BBEA-5329448F88C7}">
+          <x14:cfRule type="dataBar" id="{D190B475-D8BD-4962-B6A5-413616CFB2B1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{98E7BD88-188A-460A-9BB9-C15A4B7456EA}</x14:id>
+          <x14:id>{31674783-BB59-4923-BB67-9C339226E9AC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{70DC13FA-3455-4DFA-9EC5-59D56846EB68}</x14:id>
+          <x14:id>{39BC953D-55F7-4507-96D0-8AB63FE07416}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{62DD2A53-1661-4128-BCB8-73284A9CC0FB}</x14:id>
+          <x14:id>{1AEE65D4-7783-48AD-9E69-3BC052ECD4DD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{87470643-D778-4DD7-A43F-0F9AA20F3131}</x14:id>
+          <x14:id>{AA6AFA9F-F1FE-49CB-8521-FE821BDF7232}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{98E7BD88-188A-460A-9BB9-C15A4B7456EA}">
+          <x14:cfRule type="dataBar" id="{31674783-BB59-4923-BB67-9C339226E9AC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{70DC13FA-3455-4DFA-9EC5-59D56846EB68}">
+          <x14:cfRule type="dataBar" id="{39BC953D-55F7-4507-96D0-8AB63FE07416}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{62DD2A53-1661-4128-BCB8-73284A9CC0FB}">
+          <x14:cfRule type="dataBar" id="{1AEE65D4-7783-48AD-9E69-3BC052ECD4DD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{87470643-D778-4DD7-A43F-0F9AA20F3131}">
+          <x14:cfRule type="dataBar" id="{AA6AFA9F-F1FE-49CB-8521-FE821BDF7232}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5250E87C-DB5F-49E7-9FAD-E5B100C9A403}</x14:id>
+          <x14:id>{2ABE8926-BA78-4B4C-B610-B4830C2B56EF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C39CBEF7-CCA3-4D5C-8D1D-302310DB5396}</x14:id>
+          <x14:id>{F5EDDF16-20CC-44A7-A390-C18A246596C5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{63A4C655-CD3E-483D-90B2-DE0665E8E510}</x14:id>
+          <x14:id>{2124AB3A-CE5A-4AD8-B977-4FE5F3126A34}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D190B475-D8BD-4962-B6A5-413616CFB2B1}</x14:id>
+          <x14:id>{960E0C40-95F4-4E4A-A221-0FA5B0DD62D6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5250E87C-DB5F-49E7-9FAD-E5B100C9A403}">
+          <x14:cfRule type="dataBar" id="{2ABE8926-BA78-4B4C-B610-B4830C2B56EF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C39CBEF7-CCA3-4D5C-8D1D-302310DB5396}">
+          <x14:cfRule type="dataBar" id="{F5EDDF16-20CC-44A7-A390-C18A246596C5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{63A4C655-CD3E-483D-90B2-DE0665E8E510}">
+          <x14:cfRule type="dataBar" id="{2124AB3A-CE5A-4AD8-B977-4FE5F3126A34}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D190B475-D8BD-4962-B6A5-413616CFB2B1}">
+          <x14:cfRule type="dataBar" id="{960E0C40-95F4-4E4A-A221-0FA5B0DD62D6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{31674783-BB59-4923-BB67-9C339226E9AC}</x14:id>
+          <x14:id>{1EA78870-8F33-4C89-B812-F64E9708F154}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{39BC953D-55F7-4507-96D0-8AB63FE07416}</x14:id>
+          <x14:id>{D6C2AA29-9670-4782-8BAD-5FB35DC4FCD6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1AEE65D4-7783-48AD-9E69-3BC052ECD4DD}</x14:id>
+          <x14:id>{6FAC15A6-C1B0-4202-A96F-A26161F5FB94}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AA6AFA9F-F1FE-49CB-8521-FE821BDF7232}</x14:id>
+          <x14:id>{1E5472B3-2329-439B-B708-D1728D936377}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{31674783-BB59-4923-BB67-9C339226E9AC}">
+          <x14:cfRule type="dataBar" id="{1EA78870-8F33-4C89-B812-F64E9708F154}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{39BC953D-55F7-4507-96D0-8AB63FE07416}">
+          <x14:cfRule type="dataBar" id="{D6C2AA29-9670-4782-8BAD-5FB35DC4FCD6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1AEE65D4-7783-48AD-9E69-3BC052ECD4DD}">
+          <x14:cfRule type="dataBar" id="{6FAC15A6-C1B0-4202-A96F-A26161F5FB94}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AA6AFA9F-F1FE-49CB-8521-FE821BDF7232}">
+          <x14:cfRule type="dataBar" id="{1E5472B3-2329-439B-B708-D1728D936377}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2ABE8926-BA78-4B4C-B610-B4830C2B56EF}</x14:id>
+          <x14:id>{1541B454-728E-465F-83C1-55BA61287273}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F5EDDF16-20CC-44A7-A390-C18A246596C5}</x14:id>
+          <x14:id>{7052BDAA-A856-44DE-A9D7-59941AADE998}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2124AB3A-CE5A-4AD8-B977-4FE5F3126A34}</x14:id>
+          <x14:id>{F4FCC347-5F55-4BAE-9E8F-E42CBB7AF682}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{960E0C40-95F4-4E4A-A221-0FA5B0DD62D6}</x14:id>
+          <x14:id>{E8B4EB08-C3AF-42AD-AAA2-02E28FABEDFC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2ABE8926-BA78-4B4C-B610-B4830C2B56EF}">
+          <x14:cfRule type="dataBar" id="{1541B454-728E-465F-83C1-55BA61287273}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F5EDDF16-20CC-44A7-A390-C18A246596C5}">
+          <x14:cfRule type="dataBar" id="{7052BDAA-A856-44DE-A9D7-59941AADE998}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2124AB3A-CE5A-4AD8-B977-4FE5F3126A34}">
+          <x14:cfRule type="dataBar" id="{F4FCC347-5F55-4BAE-9E8F-E42CBB7AF682}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{960E0C40-95F4-4E4A-A221-0FA5B0DD62D6}">
+          <x14:cfRule type="dataBar" id="{E8B4EB08-C3AF-42AD-AAA2-02E28FABEDFC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1EA78870-8F33-4C89-B812-F64E9708F154}</x14:id>
+          <x14:id>{A16DCBF1-4BDB-42F8-8F10-61650D0E9C74}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D6C2AA29-9670-4782-8BAD-5FB35DC4FCD6}</x14:id>
+          <x14:id>{1073A40B-5390-4F5D-A535-47C7AA963423}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6FAC15A6-C1B0-4202-A96F-A26161F5FB94}</x14:id>
+          <x14:id>{8CB07EB6-CB6D-46F3-AE4F-0932A70593B8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1E5472B3-2329-439B-B708-D1728D936377}</x14:id>
+          <x14:id>{EEFD053E-C5BB-476B-82F0-4D1432B1A1C1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1EA78870-8F33-4C89-B812-F64E9708F154}">
+          <x14:cfRule type="dataBar" id="{A16DCBF1-4BDB-42F8-8F10-61650D0E9C74}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D6C2AA29-9670-4782-8BAD-5FB35DC4FCD6}">
+          <x14:cfRule type="dataBar" id="{1073A40B-5390-4F5D-A535-47C7AA963423}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6FAC15A6-C1B0-4202-A96F-A26161F5FB94}">
+          <x14:cfRule type="dataBar" id="{8CB07EB6-CB6D-46F3-AE4F-0932A70593B8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1E5472B3-2329-439B-B708-D1728D936377}">
+          <x14:cfRule type="dataBar" id="{EEFD053E-C5BB-476B-82F0-4D1432B1A1C1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1541B454-728E-465F-83C1-55BA61287273}</x14:id>
+          <x14:id>{BCDFC655-D427-4EDD-A48D-1B92FC826AC7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7052BDAA-A856-44DE-A9D7-59941AADE998}</x14:id>
+          <x14:id>{C99A131C-DB57-4F25-AAC2-03F4B6FAB710}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F4FCC347-5F55-4BAE-9E8F-E42CBB7AF682}</x14:id>
+          <x14:id>{E933FA4A-109B-49C3-8804-B10F72E167C3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E8B4EB08-C3AF-42AD-AAA2-02E28FABEDFC}</x14:id>
+          <x14:id>{52380E76-64DF-41F7-BAF0-CC192E02E774}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1541B454-728E-465F-83C1-55BA61287273}">
+          <x14:cfRule type="dataBar" id="{BCDFC655-D427-4EDD-A48D-1B92FC826AC7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7052BDAA-A856-44DE-A9D7-59941AADE998}">
+          <x14:cfRule type="dataBar" id="{C99A131C-DB57-4F25-AAC2-03F4B6FAB710}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F4FCC347-5F55-4BAE-9E8F-E42CBB7AF682}">
+          <x14:cfRule type="dataBar" id="{E933FA4A-109B-49C3-8804-B10F72E167C3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E8B4EB08-C3AF-42AD-AAA2-02E28FABEDFC}">
+          <x14:cfRule type="dataBar" id="{52380E76-64DF-41F7-BAF0-CC192E02E774}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A16DCBF1-4BDB-42F8-8F10-61650D0E9C74}</x14:id>
+          <x14:id>{FE2C0364-A010-476D-A776-5B140032F236}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1073A40B-5390-4F5D-A535-47C7AA963423}</x14:id>
+          <x14:id>{EA14EA85-B9DA-4A32-BE3A-684438FB9C60}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8CB07EB6-CB6D-46F3-AE4F-0932A70593B8}</x14:id>
+          <x14:id>{B638837B-D7A7-4A83-BFAA-37FA0E5A9099}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EEFD053E-C5BB-476B-82F0-4D1432B1A1C1}</x14:id>
+          <x14:id>{7A0DBA34-EBB2-460D-896C-656CA0C0AC7E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A16DCBF1-4BDB-42F8-8F10-61650D0E9C74}">
+          <x14:cfRule type="dataBar" id="{FE2C0364-A010-476D-A776-5B140032F236}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1073A40B-5390-4F5D-A535-47C7AA963423}">
+          <x14:cfRule type="dataBar" id="{EA14EA85-B9DA-4A32-BE3A-684438FB9C60}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8CB07EB6-CB6D-46F3-AE4F-0932A70593B8}">
+          <x14:cfRule type="dataBar" id="{B638837B-D7A7-4A83-BFAA-37FA0E5A9099}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EEFD053E-C5BB-476B-82F0-4D1432B1A1C1}">
+          <x14:cfRule type="dataBar" id="{7A0DBA34-EBB2-460D-896C-656CA0C0AC7E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BCDFC655-D427-4EDD-A48D-1B92FC826AC7}</x14:id>
+          <x14:id>{D9545ABA-D25C-47F8-A50C-0AB1AD421786}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C99A131C-DB57-4F25-AAC2-03F4B6FAB710}</x14:id>
+          <x14:id>{BEC57434-8710-498F-A398-CFCB7436F921}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E933FA4A-109B-49C3-8804-B10F72E167C3}</x14:id>
+          <x14:id>{A38A802E-A591-422F-8996-A5A9B89C1F7D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{52380E76-64DF-41F7-BAF0-CC192E02E774}</x14:id>
+          <x14:id>{57A923E7-7CE2-4CFF-9A5E-25411B6F4705}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BCDFC655-D427-4EDD-A48D-1B92FC826AC7}">
+          <x14:cfRule type="dataBar" id="{D9545ABA-D25C-47F8-A50C-0AB1AD421786}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C99A131C-DB57-4F25-AAC2-03F4B6FAB710}">
+          <x14:cfRule type="dataBar" id="{BEC57434-8710-498F-A398-CFCB7436F921}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E933FA4A-109B-49C3-8804-B10F72E167C3}">
+          <x14:cfRule type="dataBar" id="{A38A802E-A591-422F-8996-A5A9B89C1F7D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{52380E76-64DF-41F7-BAF0-CC192E02E774}">
+          <x14:cfRule type="dataBar" id="{57A923E7-7CE2-4CFF-9A5E-25411B6F4705}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FE2C0364-A010-476D-A776-5B140032F236}</x14:id>
+          <x14:id>{FB5E4636-BE8D-4553-9B84-D9E8320F85C8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EA14EA85-B9DA-4A32-BE3A-684438FB9C60}</x14:id>
+          <x14:id>{FBFE4876-5BEE-4579-9314-4C4B44D56383}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B638837B-D7A7-4A83-BFAA-37FA0E5A9099}</x14:id>
+          <x14:id>{59527F4D-0696-4529-AFBB-C45FEA099D5B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7A0DBA34-EBB2-460D-896C-656CA0C0AC7E}</x14:id>
+          <x14:id>{6D00D24C-3AFF-45D0-B841-591248E8F750}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FE2C0364-A010-476D-A776-5B140032F236}">
+          <x14:cfRule type="dataBar" id="{FB5E4636-BE8D-4553-9B84-D9E8320F85C8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EA14EA85-B9DA-4A32-BE3A-684438FB9C60}">
+          <x14:cfRule type="dataBar" id="{FBFE4876-5BEE-4579-9314-4C4B44D56383}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B638837B-D7A7-4A83-BFAA-37FA0E5A9099}">
+          <x14:cfRule type="dataBar" id="{59527F4D-0696-4529-AFBB-C45FEA099D5B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7A0DBA34-EBB2-460D-896C-656CA0C0AC7E}">
+          <x14:cfRule type="dataBar" id="{6D00D24C-3AFF-45D0-B841-591248E8F750}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D9545ABA-D25C-47F8-A50C-0AB1AD421786}</x14:id>
+          <x14:id>{17040BCD-A466-41F3-9DF2-AD9BD8B6744D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BEC57434-8710-498F-A398-CFCB7436F921}</x14:id>
+          <x14:id>{4CB7393F-73EC-46EC-A1E8-04EA3D18C628}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A38A802E-A591-422F-8996-A5A9B89C1F7D}</x14:id>
+          <x14:id>{3FCC91CB-297B-4254-BA47-069E5527FF04}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{57A923E7-7CE2-4CFF-9A5E-25411B6F4705}</x14:id>
+          <x14:id>{D6629F08-116A-4397-8464-43C080118648}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D9545ABA-D25C-47F8-A50C-0AB1AD421786}">
+          <x14:cfRule type="dataBar" id="{17040BCD-A466-41F3-9DF2-AD9BD8B6744D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BEC57434-8710-498F-A398-CFCB7436F921}">
+          <x14:cfRule type="dataBar" id="{4CB7393F-73EC-46EC-A1E8-04EA3D18C628}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A38A802E-A591-422F-8996-A5A9B89C1F7D}">
+          <x14:cfRule type="dataBar" id="{3FCC91CB-297B-4254-BA47-069E5527FF04}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{57A923E7-7CE2-4CFF-9A5E-25411B6F4705}">
+          <x14:cfRule type="dataBar" id="{D6629F08-116A-4397-8464-43C080118648}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FB5E4636-BE8D-4553-9B84-D9E8320F85C8}</x14:id>
+          <x14:id>{A4DE690D-53E4-43DB-B144-2699466C5633}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FBFE4876-5BEE-4579-9314-4C4B44D56383}</x14:id>
+          <x14:id>{125720DA-6A6B-4E00-B1DB-F6473861953A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{59527F4D-0696-4529-AFBB-C45FEA099D5B}</x14:id>
+          <x14:id>{3FAA87B6-2EFF-4D64-9D00-FD2E763227EE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6D00D24C-3AFF-45D0-B841-591248E8F750}</x14:id>
+          <x14:id>{146F30DD-74B1-4E1A-B584-349EA925D9E9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FB5E4636-BE8D-4553-9B84-D9E8320F85C8}">
+          <x14:cfRule type="dataBar" id="{A4DE690D-53E4-43DB-B144-2699466C5633}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FBFE4876-5BEE-4579-9314-4C4B44D56383}">
+          <x14:cfRule type="dataBar" id="{125720DA-6A6B-4E00-B1DB-F6473861953A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{59527F4D-0696-4529-AFBB-C45FEA099D5B}">
+          <x14:cfRule type="dataBar" id="{3FAA87B6-2EFF-4D64-9D00-FD2E763227EE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6D00D24C-3AFF-45D0-B841-591248E8F750}">
+          <x14:cfRule type="dataBar" id="{146F30DD-74B1-4E1A-B584-349EA925D9E9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{17040BCD-A466-41F3-9DF2-AD9BD8B6744D}</x14:id>
+          <x14:id>{89582B36-4DC5-4665-85AD-2105F1A62F56}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4CB7393F-73EC-46EC-A1E8-04EA3D18C628}</x14:id>
+          <x14:id>{98001F74-650C-416A-887F-E2B228AEC1C9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3FCC91CB-297B-4254-BA47-069E5527FF04}</x14:id>
+          <x14:id>{C2DD0A97-3272-49DA-A215-D162BB8A5AA7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D6629F08-116A-4397-8464-43C080118648}</x14:id>
+          <x14:id>{0ACABB88-06AF-4AE0-ACB8-EAF03984D470}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{17040BCD-A466-41F3-9DF2-AD9BD8B6744D}">
+          <x14:cfRule type="dataBar" id="{89582B36-4DC5-4665-85AD-2105F1A62F56}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4CB7393F-73EC-46EC-A1E8-04EA3D18C628}">
+          <x14:cfRule type="dataBar" id="{98001F74-650C-416A-887F-E2B228AEC1C9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3FCC91CB-297B-4254-BA47-069E5527FF04}">
+          <x14:cfRule type="dataBar" id="{C2DD0A97-3272-49DA-A215-D162BB8A5AA7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D6629F08-116A-4397-8464-43C080118648}">
+          <x14:cfRule type="dataBar" id="{0ACABB88-06AF-4AE0-ACB8-EAF03984D470}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A4DE690D-53E4-43DB-B144-2699466C5633}</x14:id>
+          <x14:id>{849FADDB-0EB6-466F-B47F-5236CE525A35}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{125720DA-6A6B-4E00-B1DB-F6473861953A}</x14:id>
+          <x14:id>{EF3B95A6-47F9-4409-9749-9D342DCD9533}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3FAA87B6-2EFF-4D64-9D00-FD2E763227EE}</x14:id>
+          <x14:id>{C496ED73-BE8B-48BA-AA8D-4FB8C7D1F2EE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{146F30DD-74B1-4E1A-B584-349EA925D9E9}</x14:id>
+          <x14:id>{0BE5750D-423B-430C-9DE6-46634781488B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A4DE690D-53E4-43DB-B144-2699466C5633}">
+          <x14:cfRule type="dataBar" id="{849FADDB-0EB6-466F-B47F-5236CE525A35}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{125720DA-6A6B-4E00-B1DB-F6473861953A}">
+          <x14:cfRule type="dataBar" id="{EF3B95A6-47F9-4409-9749-9D342DCD9533}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3FAA87B6-2EFF-4D64-9D00-FD2E763227EE}">
+          <x14:cfRule type="dataBar" id="{C496ED73-BE8B-48BA-AA8D-4FB8C7D1F2EE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{146F30DD-74B1-4E1A-B584-349EA925D9E9}">
+          <x14:cfRule type="dataBar" id="{0BE5750D-423B-430C-9DE6-46634781488B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{89582B36-4DC5-4665-85AD-2105F1A62F56}</x14:id>
+          <x14:id>{73550DEE-35F9-480F-85FB-B34BD7CA77F0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{98001F74-650C-416A-887F-E2B228AEC1C9}</x14:id>
+          <x14:id>{2802208F-EE66-4CB9-A173-9075D938C1D2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C2DD0A97-3272-49DA-A215-D162BB8A5AA7}</x14:id>
+          <x14:id>{35E2A3CF-BEDE-40FE-A997-90FC2B975894}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0ACABB88-06AF-4AE0-ACB8-EAF03984D470}</x14:id>
+          <x14:id>{013B799F-DD9F-40DB-89D5-C367F8397448}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{89582B36-4DC5-4665-85AD-2105F1A62F56}">
+          <x14:cfRule type="dataBar" id="{73550DEE-35F9-480F-85FB-B34BD7CA77F0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{98001F74-650C-416A-887F-E2B228AEC1C9}">
+          <x14:cfRule type="dataBar" id="{2802208F-EE66-4CB9-A173-9075D938C1D2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C2DD0A97-3272-49DA-A215-D162BB8A5AA7}">
+          <x14:cfRule type="dataBar" id="{35E2A3CF-BEDE-40FE-A997-90FC2B975894}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0ACABB88-06AF-4AE0-ACB8-EAF03984D470}">
+          <x14:cfRule type="dataBar" id="{013B799F-DD9F-40DB-89D5-C367F8397448}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{849FADDB-0EB6-466F-B47F-5236CE525A35}</x14:id>
+          <x14:id>{78AAF4DD-BB8E-4A61-B04E-07D770C5A231}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EF3B95A6-47F9-4409-9749-9D342DCD9533}</x14:id>
+          <x14:id>{70275CE7-2451-4E91-86B3-01C94880F7FB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C496ED73-BE8B-48BA-AA8D-4FB8C7D1F2EE}</x14:id>
+          <x14:id>{359F5E46-BA08-473E-B316-A3717E806230}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0BE5750D-423B-430C-9DE6-46634781488B}</x14:id>
+          <x14:id>{0D31C189-9B37-48C4-8CDA-9DADB7D84988}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{849FADDB-0EB6-466F-B47F-5236CE525A35}">
+          <x14:cfRule type="dataBar" id="{78AAF4DD-BB8E-4A61-B04E-07D770C5A231}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EF3B95A6-47F9-4409-9749-9D342DCD9533}">
+          <x14:cfRule type="dataBar" id="{70275CE7-2451-4E91-86B3-01C94880F7FB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C496ED73-BE8B-48BA-AA8D-4FB8C7D1F2EE}">
+          <x14:cfRule type="dataBar" id="{359F5E46-BA08-473E-B316-A3717E806230}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0BE5750D-423B-430C-9DE6-46634781488B}">
+          <x14:cfRule type="dataBar" id="{0D31C189-9B37-48C4-8CDA-9DADB7D84988}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{73550DEE-35F9-480F-85FB-B34BD7CA77F0}</x14:id>
+          <x14:id>{ADCF781C-40EC-48C0-A528-83D5F64BFCC3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2802208F-EE66-4CB9-A173-9075D938C1D2}</x14:id>
+          <x14:id>{60B87CBF-3E09-4971-8988-0B16485AA7F6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{35E2A3CF-BEDE-40FE-A997-90FC2B975894}</x14:id>
+          <x14:id>{79274953-54BE-41B1-9F68-0D2AF7EC5652}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{013B799F-DD9F-40DB-89D5-C367F8397448}</x14:id>
+          <x14:id>{A126DAD8-1BEC-467C-A742-6EDE1808E2B4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{73550DEE-35F9-480F-85FB-B34BD7CA77F0}">
+          <x14:cfRule type="dataBar" id="{ADCF781C-40EC-48C0-A528-83D5F64BFCC3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2802208F-EE66-4CB9-A173-9075D938C1D2}">
+          <x14:cfRule type="dataBar" id="{60B87CBF-3E09-4971-8988-0B16485AA7F6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{35E2A3CF-BEDE-40FE-A997-90FC2B975894}">
+          <x14:cfRule type="dataBar" id="{79274953-54BE-41B1-9F68-0D2AF7EC5652}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{013B799F-DD9F-40DB-89D5-C367F8397448}">
+          <x14:cfRule type="dataBar" id="{A126DAD8-1BEC-467C-A742-6EDE1808E2B4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{78AAF4DD-BB8E-4A61-B04E-07D770C5A231}</x14:id>
+          <x14:id>{95677E37-73F5-4D4C-B1DB-838C0CE53DA9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{70275CE7-2451-4E91-86B3-01C94880F7FB}</x14:id>
+          <x14:id>{C25E5310-C577-468B-ADAF-ED78FAF9C07C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{359F5E46-BA08-473E-B316-A3717E806230}</x14:id>
+          <x14:id>{3245EEBB-38E2-4D43-B4B7-87831C440DCD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0D31C189-9B37-48C4-8CDA-9DADB7D84988}</x14:id>
+          <x14:id>{74C65EE8-8ACF-492D-BEE8-EB99FE68810C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{78AAF4DD-BB8E-4A61-B04E-07D770C5A231}">
+          <x14:cfRule type="dataBar" id="{95677E37-73F5-4D4C-B1DB-838C0CE53DA9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{70275CE7-2451-4E91-86B3-01C94880F7FB}">
+          <x14:cfRule type="dataBar" id="{C25E5310-C577-468B-ADAF-ED78FAF9C07C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{359F5E46-BA08-473E-B316-A3717E806230}">
+          <x14:cfRule type="dataBar" id="{3245EEBB-38E2-4D43-B4B7-87831C440DCD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0D31C189-9B37-48C4-8CDA-9DADB7D84988}">
+          <x14:cfRule type="dataBar" id="{74C65EE8-8ACF-492D-BEE8-EB99FE68810C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ADCF781C-40EC-48C0-A528-83D5F64BFCC3}</x14:id>
+          <x14:id>{62ED5379-1216-43E8-A263-552C69A53064}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{60B87CBF-3E09-4971-8988-0B16485AA7F6}</x14:id>
+          <x14:id>{C989AEC3-8771-40C6-A52C-7EEAAF39A6B4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{79274953-54BE-41B1-9F68-0D2AF7EC5652}</x14:id>
+          <x14:id>{0566A908-F130-4D3D-A1A3-282FE5FB1012}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A126DAD8-1BEC-467C-A742-6EDE1808E2B4}</x14:id>
+          <x14:id>{07D0DDB5-302E-4843-866F-723D8A07A397}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ADCF781C-40EC-48C0-A528-83D5F64BFCC3}">
+          <x14:cfRule type="dataBar" id="{62ED5379-1216-43E8-A263-552C69A53064}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{60B87CBF-3E09-4971-8988-0B16485AA7F6}">
+          <x14:cfRule type="dataBar" id="{C989AEC3-8771-40C6-A52C-7EEAAF39A6B4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{79274953-54BE-41B1-9F68-0D2AF7EC5652}">
+          <x14:cfRule type="dataBar" id="{0566A908-F130-4D3D-A1A3-282FE5FB1012}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A126DAD8-1BEC-467C-A742-6EDE1808E2B4}">
+          <x14:cfRule type="dataBar" id="{07D0DDB5-302E-4843-866F-723D8A07A397}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{95677E37-73F5-4D4C-B1DB-838C0CE53DA9}</x14:id>
+          <x14:id>{0A38D5F7-61AE-4048-9374-E49A9E2031E4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C25E5310-C577-468B-ADAF-ED78FAF9C07C}</x14:id>
+          <x14:id>{663E68B0-FFD9-4AB0-80BF-700A27827804}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3245EEBB-38E2-4D43-B4B7-87831C440DCD}</x14:id>
+          <x14:id>{AF1B1769-FF8F-4111-9E11-BF1645A5AE2E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{74C65EE8-8ACF-492D-BEE8-EB99FE68810C}</x14:id>
+          <x14:id>{C1D5DF31-0E75-4858-B467-D97359384650}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{95677E37-73F5-4D4C-B1DB-838C0CE53DA9}">
+          <x14:cfRule type="dataBar" id="{0A38D5F7-61AE-4048-9374-E49A9E2031E4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C25E5310-C577-468B-ADAF-ED78FAF9C07C}">
+          <x14:cfRule type="dataBar" id="{663E68B0-FFD9-4AB0-80BF-700A27827804}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3245EEBB-38E2-4D43-B4B7-87831C440DCD}">
+          <x14:cfRule type="dataBar" id="{AF1B1769-FF8F-4111-9E11-BF1645A5AE2E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{74C65EE8-8ACF-492D-BEE8-EB99FE68810C}">
+          <x14:cfRule type="dataBar" id="{C1D5DF31-0E75-4858-B467-D97359384650}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{62ED5379-1216-43E8-A263-552C69A53064}</x14:id>
+          <x14:id>{4F359223-8151-4BCD-8D2F-F7CA32B05426}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C989AEC3-8771-40C6-A52C-7EEAAF39A6B4}</x14:id>
+          <x14:id>{00B3D785-5B9C-44BD-AFD3-8B1578FE2952}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0566A908-F130-4D3D-A1A3-282FE5FB1012}</x14:id>
+          <x14:id>{0146353B-C9A9-486D-B169-377485000A9F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{07D0DDB5-302E-4843-866F-723D8A07A397}</x14:id>
+          <x14:id>{B8467D51-490F-4688-9388-E48DF878B01B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{62ED5379-1216-43E8-A263-552C69A53064}">
+          <x14:cfRule type="dataBar" id="{4F359223-8151-4BCD-8D2F-F7CA32B05426}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C989AEC3-8771-40C6-A52C-7EEAAF39A6B4}">
+          <x14:cfRule type="dataBar" id="{00B3D785-5B9C-44BD-AFD3-8B1578FE2952}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0566A908-F130-4D3D-A1A3-282FE5FB1012}">
+          <x14:cfRule type="dataBar" id="{0146353B-C9A9-486D-B169-377485000A9F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{07D0DDB5-302E-4843-866F-723D8A07A397}">
+          <x14:cfRule type="dataBar" id="{B8467D51-490F-4688-9388-E48DF878B01B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0A38D5F7-61AE-4048-9374-E49A9E2031E4}</x14:id>
+          <x14:id>{49008D50-BFAE-4839-8E52-C6F2C5C19382}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{663E68B0-FFD9-4AB0-80BF-700A27827804}</x14:id>
+          <x14:id>{2BD56FE3-B28E-4DFF-A953-8003D8C31A2A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AF1B1769-FF8F-4111-9E11-BF1645A5AE2E}</x14:id>
+          <x14:id>{B7D9E2A5-7143-45FB-8ED4-7E2C8B0F4F23}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C1D5DF31-0E75-4858-B467-D97359384650}</x14:id>
+          <x14:id>{88D36CAD-A542-456A-80A8-3A356715B07E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0A38D5F7-61AE-4048-9374-E49A9E2031E4}">
+          <x14:cfRule type="dataBar" id="{49008D50-BFAE-4839-8E52-C6F2C5C19382}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{663E68B0-FFD9-4AB0-80BF-700A27827804}">
+          <x14:cfRule type="dataBar" id="{2BD56FE3-B28E-4DFF-A953-8003D8C31A2A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AF1B1769-FF8F-4111-9E11-BF1645A5AE2E}">
+          <x14:cfRule type="dataBar" id="{B7D9E2A5-7143-45FB-8ED4-7E2C8B0F4F23}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C1D5DF31-0E75-4858-B467-D97359384650}">
+          <x14:cfRule type="dataBar" id="{88D36CAD-A542-456A-80A8-3A356715B07E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4F359223-8151-4BCD-8D2F-F7CA32B05426}</x14:id>
+          <x14:id>{CD73D994-F7D8-4BA0-8505-3143862147DD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{00B3D785-5B9C-44BD-AFD3-8B1578FE2952}</x14:id>
+          <x14:id>{07DC8210-AEFA-4ACD-9F61-4AB08A753A0B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0146353B-C9A9-486D-B169-377485000A9F}</x14:id>
+          <x14:id>{F047DBDD-D6AA-410A-996C-A34C43EA2EEE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B8467D51-490F-4688-9388-E48DF878B01B}</x14:id>
+          <x14:id>{9445B4F2-7627-4C17-B980-738A0EB50E62}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4F359223-8151-4BCD-8D2F-F7CA32B05426}">
+          <x14:cfRule type="dataBar" id="{CD73D994-F7D8-4BA0-8505-3143862147DD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{00B3D785-5B9C-44BD-AFD3-8B1578FE2952}">
+          <x14:cfRule type="dataBar" id="{07DC8210-AEFA-4ACD-9F61-4AB08A753A0B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0146353B-C9A9-486D-B169-377485000A9F}">
+          <x14:cfRule type="dataBar" id="{F047DBDD-D6AA-410A-996C-A34C43EA2EEE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B8467D51-490F-4688-9388-E48DF878B01B}">
+          <x14:cfRule type="dataBar" id="{9445B4F2-7627-4C17-B980-738A0EB50E62}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-19 09:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -10678,7 +10678,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49008D50-BFAE-4839-8E52-C6F2C5C19382}</x14:id>
+          <x14:id>{7D339DA7-81D3-46EA-B7B3-D32D8D378822}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10692,7 +10692,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2BD56FE3-B28E-4DFF-A953-8003D8C31A2A}</x14:id>
+          <x14:id>{A85D765B-331B-4B9D-841F-C285CC0D0313}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10706,7 +10706,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B7D9E2A5-7143-45FB-8ED4-7E2C8B0F4F23}</x14:id>
+          <x14:id>{40036C0D-DC43-4BF1-87C8-5CBCA690AB6A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10720,7 +10720,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{88D36CAD-A542-456A-80A8-3A356715B07E}</x14:id>
+          <x14:id>{76E7CF6A-06C6-421F-A53A-71815930644E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10730,7 +10730,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49008D50-BFAE-4839-8E52-C6F2C5C19382}">
+          <x14:cfRule type="dataBar" id="{7D339DA7-81D3-46EA-B7B3-D32D8D378822}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10743,7 +10743,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2BD56FE3-B28E-4DFF-A953-8003D8C31A2A}">
+          <x14:cfRule type="dataBar" id="{A85D765B-331B-4B9D-841F-C285CC0D0313}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10756,7 +10756,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B7D9E2A5-7143-45FB-8ED4-7E2C8B0F4F23}">
+          <x14:cfRule type="dataBar" id="{40036C0D-DC43-4BF1-87C8-5CBCA690AB6A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10769,7 +10769,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{88D36CAD-A542-456A-80A8-3A356715B07E}">
+          <x14:cfRule type="dataBar" id="{76E7CF6A-06C6-421F-A53A-71815930644E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26063,7 +26063,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CD73D994-F7D8-4BA0-8505-3143862147DD}</x14:id>
+          <x14:id>{E99193B8-0B93-410C-AC40-994C94FC31AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26077,7 +26077,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{07DC8210-AEFA-4ACD-9F61-4AB08A753A0B}</x14:id>
+          <x14:id>{E245563E-26B8-41C4-B3B2-11A15B22CE40}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26091,7 +26091,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F047DBDD-D6AA-410A-996C-A34C43EA2EEE}</x14:id>
+          <x14:id>{B6FDA0A3-B40E-4B56-8790-41DCCC58E90E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26105,7 +26105,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9445B4F2-7627-4C17-B980-738A0EB50E62}</x14:id>
+          <x14:id>{6A7676A2-BACF-4C14-A9E4-93175FAF44A9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26115,7 +26115,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CD73D994-F7D8-4BA0-8505-3143862147DD}">
+          <x14:cfRule type="dataBar" id="{E99193B8-0B93-410C-AC40-994C94FC31AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26128,7 +26128,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{07DC8210-AEFA-4ACD-9F61-4AB08A753A0B}">
+          <x14:cfRule type="dataBar" id="{E245563E-26B8-41C4-B3B2-11A15B22CE40}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26141,7 +26141,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F047DBDD-D6AA-410A-996C-A34C43EA2EEE}">
+          <x14:cfRule type="dataBar" id="{B6FDA0A3-B40E-4B56-8790-41DCCC58E90E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26154,7 +26154,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9445B4F2-7627-4C17-B980-738A0EB50E62}">
+          <x14:cfRule type="dataBar" id="{6A7676A2-BACF-4C14-A9E4-93175FAF44A9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-20 07:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -11484,7 +11484,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C7DBC3D1-55DB-4E5C-8D28-961FCB0C8BE5}</x14:id>
+          <x14:id>{20C09BE8-16F4-4123-8150-A69FFD303F65}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11498,7 +11498,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FFF34066-FD1C-4EFC-8E59-F961894CD349}</x14:id>
+          <x14:id>{25C4B3CE-9906-44B1-A9C1-9FE58D0630A6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11512,7 +11512,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A527E2BA-97B2-4436-BF67-E95BC54EEB61}</x14:id>
+          <x14:id>{55490AC3-4A7E-438E-A19A-781937F84A64}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11526,7 +11526,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{991C0332-8806-4726-B91F-3F43D6238E4B}</x14:id>
+          <x14:id>{67E988F5-9F3D-44BB-89E2-D60313EC18D0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11536,7 +11536,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C7DBC3D1-55DB-4E5C-8D28-961FCB0C8BE5}">
+          <x14:cfRule type="dataBar" id="{20C09BE8-16F4-4123-8150-A69FFD303F65}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11549,7 +11549,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FFF34066-FD1C-4EFC-8E59-F961894CD349}">
+          <x14:cfRule type="dataBar" id="{25C4B3CE-9906-44B1-A9C1-9FE58D0630A6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11562,7 +11562,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A527E2BA-97B2-4436-BF67-E95BC54EEB61}">
+          <x14:cfRule type="dataBar" id="{55490AC3-4A7E-438E-A19A-781937F84A64}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11575,7 +11575,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{991C0332-8806-4726-B91F-3F43D6238E4B}">
+          <x14:cfRule type="dataBar" id="{67E988F5-9F3D-44BB-89E2-D60313EC18D0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26835,7 +26835,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2C5B2C38-EE61-4D31-BA26-A30699ED7AC8}</x14:id>
+          <x14:id>{FF345574-1C96-47FE-B0A6-21C7600CCD2A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26849,7 +26849,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{79CF5D6C-1DD3-4AFF-9412-9FB9AB2B736B}</x14:id>
+          <x14:id>{1E5F4F77-65E0-4613-A794-88B74A63477C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26863,7 +26863,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{599E1C1F-8753-4541-BA9E-36E0981DF340}</x14:id>
+          <x14:id>{7D6E2EC2-D254-4917-956F-FA8FCE356B28}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26877,7 +26877,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E02182C6-FFA3-4E04-AA43-9EA82C11A00D}</x14:id>
+          <x14:id>{2FE7C92C-C8A5-4345-966D-D27BBB054F78}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -26887,7 +26887,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2C5B2C38-EE61-4D31-BA26-A30699ED7AC8}">
+          <x14:cfRule type="dataBar" id="{FF345574-1C96-47FE-B0A6-21C7600CCD2A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26900,7 +26900,7 @@
           <xm:sqref>N6:N173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{79CF5D6C-1DD3-4AFF-9412-9FB9AB2B736B}">
+          <x14:cfRule type="dataBar" id="{1E5F4F77-65E0-4613-A794-88B74A63477C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26913,7 +26913,7 @@
           <xm:sqref>P6:P173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{599E1C1F-8753-4541-BA9E-36E0981DF340}">
+          <x14:cfRule type="dataBar" id="{7D6E2EC2-D254-4917-956F-FA8FCE356B28}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -26926,7 +26926,7 @@
           <xm:sqref>Y6:Y173</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E02182C6-FFA3-4E04-AA43-9EA82C11A00D}">
+          <x14:cfRule type="dataBar" id="{2FE7C92C-C8A5-4345-966D-D27BBB054F78}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 07:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F5D09EDD-B723-4804-A00D-2A8088DDDD61}</x14:id>
+          <x14:id>{C8322E8C-D8CA-4F83-8B8A-78FCF211AEAD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F31F0816-6F72-44C2-AB4C-13958BF40E32}</x14:id>
+          <x14:id>{5B2AC480-095D-4F98-A035-1108D6FB29F2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4C9F6676-7023-4932-B844-4B6AE20EB6F7}</x14:id>
+          <x14:id>{17F3C572-8425-4F8E-881D-656C45BCBA04}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{06A984CF-71C6-480C-93DC-440A8ABBD400}</x14:id>
+          <x14:id>{5C049FA0-73C9-4F6C-BDC9-E37E9C03340C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F5D09EDD-B723-4804-A00D-2A8088DDDD61}">
+          <x14:cfRule type="dataBar" id="{C8322E8C-D8CA-4F83-8B8A-78FCF211AEAD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F31F0816-6F72-44C2-AB4C-13958BF40E32}">
+          <x14:cfRule type="dataBar" id="{5B2AC480-095D-4F98-A035-1108D6FB29F2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4C9F6676-7023-4932-B844-4B6AE20EB6F7}">
+          <x14:cfRule type="dataBar" id="{17F3C572-8425-4F8E-881D-656C45BCBA04}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{06A984CF-71C6-480C-93DC-440A8ABBD400}">
+          <x14:cfRule type="dataBar" id="{5C049FA0-73C9-4F6C-BDC9-E37E9C03340C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A1FE7328-EA10-45A7-BFEF-88132CA8DB72}</x14:id>
+          <x14:id>{087F737E-44D2-49E7-8D76-9487F42C520A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{273BDE8A-2A92-45C1-9C8B-2F74A46FD97B}</x14:id>
+          <x14:id>{23208D9E-4EE7-4A55-A7A4-058D17E91E0E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7E257C9D-6CF8-41DB-81A5-3A769F457E5E}</x14:id>
+          <x14:id>{05DE294F-8538-42E2-A925-4B7C552D70F1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9450B635-8957-40E2-B05B-065B8FC3DCE9}</x14:id>
+          <x14:id>{125D8D5C-35A1-4FCA-BC15-D4CDF69038A1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A1FE7328-EA10-45A7-BFEF-88132CA8DB72}">
+          <x14:cfRule type="dataBar" id="{087F737E-44D2-49E7-8D76-9487F42C520A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{273BDE8A-2A92-45C1-9C8B-2F74A46FD97B}">
+          <x14:cfRule type="dataBar" id="{23208D9E-4EE7-4A55-A7A4-058D17E91E0E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7E257C9D-6CF8-41DB-81A5-3A769F457E5E}">
+          <x14:cfRule type="dataBar" id="{05DE294F-8538-42E2-A925-4B7C552D70F1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9450B635-8957-40E2-B05B-065B8FC3DCE9}">
+          <x14:cfRule type="dataBar" id="{125D8D5C-35A1-4FCA-BC15-D4CDF69038A1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 07:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C8322E8C-D8CA-4F83-8B8A-78FCF211AEAD}</x14:id>
+          <x14:id>{D3448BF0-6F20-4F3D-95FC-7AC59D9B152A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5B2AC480-095D-4F98-A035-1108D6FB29F2}</x14:id>
+          <x14:id>{E84E60F1-05AF-45BD-AFE1-BB9D90B097D9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{17F3C572-8425-4F8E-881D-656C45BCBA04}</x14:id>
+          <x14:id>{BD7C3EA9-E1F3-4230-8AAC-B34BEDC4F038}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5C049FA0-73C9-4F6C-BDC9-E37E9C03340C}</x14:id>
+          <x14:id>{920D4859-268C-4E88-8698-BFFAC8EA01D9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C8322E8C-D8CA-4F83-8B8A-78FCF211AEAD}">
+          <x14:cfRule type="dataBar" id="{D3448BF0-6F20-4F3D-95FC-7AC59D9B152A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5B2AC480-095D-4F98-A035-1108D6FB29F2}">
+          <x14:cfRule type="dataBar" id="{E84E60F1-05AF-45BD-AFE1-BB9D90B097D9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{17F3C572-8425-4F8E-881D-656C45BCBA04}">
+          <x14:cfRule type="dataBar" id="{BD7C3EA9-E1F3-4230-8AAC-B34BEDC4F038}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5C049FA0-73C9-4F6C-BDC9-E37E9C03340C}">
+          <x14:cfRule type="dataBar" id="{920D4859-268C-4E88-8698-BFFAC8EA01D9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{087F737E-44D2-49E7-8D76-9487F42C520A}</x14:id>
+          <x14:id>{F8D8907A-A580-4B42-8723-7F398347A767}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{23208D9E-4EE7-4A55-A7A4-058D17E91E0E}</x14:id>
+          <x14:id>{23D159CD-9E67-46E4-B101-9B98C8206C61}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{05DE294F-8538-42E2-A925-4B7C552D70F1}</x14:id>
+          <x14:id>{4DBE6239-8FE9-4344-B87A-7F3C967EBA37}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{125D8D5C-35A1-4FCA-BC15-D4CDF69038A1}</x14:id>
+          <x14:id>{DAE56C23-E092-46E0-8BC2-B1A495F77D0C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{087F737E-44D2-49E7-8D76-9487F42C520A}">
+          <x14:cfRule type="dataBar" id="{F8D8907A-A580-4B42-8723-7F398347A767}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{23208D9E-4EE7-4A55-A7A4-058D17E91E0E}">
+          <x14:cfRule type="dataBar" id="{23D159CD-9E67-46E4-B101-9B98C8206C61}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{05DE294F-8538-42E2-A925-4B7C552D70F1}">
+          <x14:cfRule type="dataBar" id="{4DBE6239-8FE9-4344-B87A-7F3C967EBA37}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{125D8D5C-35A1-4FCA-BC15-D4CDF69038A1}">
+          <x14:cfRule type="dataBar" id="{DAE56C23-E092-46E0-8BC2-B1A495F77D0C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D3448BF0-6F20-4F3D-95FC-7AC59D9B152A}</x14:id>
+          <x14:id>{230B67AC-3DDD-4644-AB23-05AD0CE4A5AD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E84E60F1-05AF-45BD-AFE1-BB9D90B097D9}</x14:id>
+          <x14:id>{49A68AD5-8EA9-486A-ABFE-884F0790BC41}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BD7C3EA9-E1F3-4230-8AAC-B34BEDC4F038}</x14:id>
+          <x14:id>{DD46DB8E-385D-4941-8AA5-9C8CAC2329EA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{920D4859-268C-4E88-8698-BFFAC8EA01D9}</x14:id>
+          <x14:id>{49478C12-446E-44AC-A310-FBED7F955357}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D3448BF0-6F20-4F3D-95FC-7AC59D9B152A}">
+          <x14:cfRule type="dataBar" id="{230B67AC-3DDD-4644-AB23-05AD0CE4A5AD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E84E60F1-05AF-45BD-AFE1-BB9D90B097D9}">
+          <x14:cfRule type="dataBar" id="{49A68AD5-8EA9-486A-ABFE-884F0790BC41}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BD7C3EA9-E1F3-4230-8AAC-B34BEDC4F038}">
+          <x14:cfRule type="dataBar" id="{DD46DB8E-385D-4941-8AA5-9C8CAC2329EA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{920D4859-268C-4E88-8698-BFFAC8EA01D9}">
+          <x14:cfRule type="dataBar" id="{49478C12-446E-44AC-A310-FBED7F955357}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F8D8907A-A580-4B42-8723-7F398347A767}</x14:id>
+          <x14:id>{CB456A0A-FD4F-4BE2-810B-D6A53FF9F7A1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{23D159CD-9E67-46E4-B101-9B98C8206C61}</x14:id>
+          <x14:id>{8F177015-18C2-4C56-8E2C-11AFFA002B63}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4DBE6239-8FE9-4344-B87A-7F3C967EBA37}</x14:id>
+          <x14:id>{F49F93C3-41C0-411F-B73B-8A8C2C348690}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DAE56C23-E092-46E0-8BC2-B1A495F77D0C}</x14:id>
+          <x14:id>{4C15792A-8C90-4710-BFCA-EA3874635495}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F8D8907A-A580-4B42-8723-7F398347A767}">
+          <x14:cfRule type="dataBar" id="{CB456A0A-FD4F-4BE2-810B-D6A53FF9F7A1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{23D159CD-9E67-46E4-B101-9B98C8206C61}">
+          <x14:cfRule type="dataBar" id="{8F177015-18C2-4C56-8E2C-11AFFA002B63}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4DBE6239-8FE9-4344-B87A-7F3C967EBA37}">
+          <x14:cfRule type="dataBar" id="{F49F93C3-41C0-411F-B73B-8A8C2C348690}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DAE56C23-E092-46E0-8BC2-B1A495F77D0C}">
+          <x14:cfRule type="dataBar" id="{4C15792A-8C90-4710-BFCA-EA3874635495}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{230B67AC-3DDD-4644-AB23-05AD0CE4A5AD}</x14:id>
+          <x14:id>{FAF1C4F8-1F71-4A3F-AAAF-7BA8549A8D1B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49A68AD5-8EA9-486A-ABFE-884F0790BC41}</x14:id>
+          <x14:id>{16718607-1515-414F-9308-B52EC0BCC94A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DD46DB8E-385D-4941-8AA5-9C8CAC2329EA}</x14:id>
+          <x14:id>{5A05E42B-4648-48C0-9A62-FAC34999A7B7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49478C12-446E-44AC-A310-FBED7F955357}</x14:id>
+          <x14:id>{0B32DD39-BB33-405B-AFCD-3792A2AEC487}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{230B67AC-3DDD-4644-AB23-05AD0CE4A5AD}">
+          <x14:cfRule type="dataBar" id="{FAF1C4F8-1F71-4A3F-AAAF-7BA8549A8D1B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49A68AD5-8EA9-486A-ABFE-884F0790BC41}">
+          <x14:cfRule type="dataBar" id="{16718607-1515-414F-9308-B52EC0BCC94A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DD46DB8E-385D-4941-8AA5-9C8CAC2329EA}">
+          <x14:cfRule type="dataBar" id="{5A05E42B-4648-48C0-9A62-FAC34999A7B7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49478C12-446E-44AC-A310-FBED7F955357}">
+          <x14:cfRule type="dataBar" id="{0B32DD39-BB33-405B-AFCD-3792A2AEC487}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CB456A0A-FD4F-4BE2-810B-D6A53FF9F7A1}</x14:id>
+          <x14:id>{154D9996-CCEC-44A4-92FD-789A7610E502}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8F177015-18C2-4C56-8E2C-11AFFA002B63}</x14:id>
+          <x14:id>{0EFD3CFD-D976-4AC2-B422-6C53A467A85B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F49F93C3-41C0-411F-B73B-8A8C2C348690}</x14:id>
+          <x14:id>{9EB5E666-0641-4274-B41A-CD6BAAD702FF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4C15792A-8C90-4710-BFCA-EA3874635495}</x14:id>
+          <x14:id>{88E62804-B35E-476D-9FE2-869194458182}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CB456A0A-FD4F-4BE2-810B-D6A53FF9F7A1}">
+          <x14:cfRule type="dataBar" id="{154D9996-CCEC-44A4-92FD-789A7610E502}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8F177015-18C2-4C56-8E2C-11AFFA002B63}">
+          <x14:cfRule type="dataBar" id="{0EFD3CFD-D976-4AC2-B422-6C53A467A85B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F49F93C3-41C0-411F-B73B-8A8C2C348690}">
+          <x14:cfRule type="dataBar" id="{9EB5E666-0641-4274-B41A-CD6BAAD702FF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4C15792A-8C90-4710-BFCA-EA3874635495}">
+          <x14:cfRule type="dataBar" id="{88E62804-B35E-476D-9FE2-869194458182}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FAF1C4F8-1F71-4A3F-AAAF-7BA8549A8D1B}</x14:id>
+          <x14:id>{4E209570-8B3A-4094-9BFE-F7C8E87A30C8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{16718607-1515-414F-9308-B52EC0BCC94A}</x14:id>
+          <x14:id>{803DFF29-392D-4BD6-A963-6EF06A3A1375}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5A05E42B-4648-48C0-9A62-FAC34999A7B7}</x14:id>
+          <x14:id>{C67F1B23-7383-42D8-97D7-B2C0105CF592}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0B32DD39-BB33-405B-AFCD-3792A2AEC487}</x14:id>
+          <x14:id>{35A53036-9160-40FF-B779-357515D8E1D2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FAF1C4F8-1F71-4A3F-AAAF-7BA8549A8D1B}">
+          <x14:cfRule type="dataBar" id="{4E209570-8B3A-4094-9BFE-F7C8E87A30C8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{16718607-1515-414F-9308-B52EC0BCC94A}">
+          <x14:cfRule type="dataBar" id="{803DFF29-392D-4BD6-A963-6EF06A3A1375}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5A05E42B-4648-48C0-9A62-FAC34999A7B7}">
+          <x14:cfRule type="dataBar" id="{C67F1B23-7383-42D8-97D7-B2C0105CF592}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0B32DD39-BB33-405B-AFCD-3792A2AEC487}">
+          <x14:cfRule type="dataBar" id="{35A53036-9160-40FF-B779-357515D8E1D2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{154D9996-CCEC-44A4-92FD-789A7610E502}</x14:id>
+          <x14:id>{822BE966-7648-49EA-A3BC-01A01B84DF94}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0EFD3CFD-D976-4AC2-B422-6C53A467A85B}</x14:id>
+          <x14:id>{9B5B630B-C2B1-4E03-9705-78BF3C53EC96}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9EB5E666-0641-4274-B41A-CD6BAAD702FF}</x14:id>
+          <x14:id>{E6437F2B-05FF-44EB-9232-AB98C280E5C5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{88E62804-B35E-476D-9FE2-869194458182}</x14:id>
+          <x14:id>{6BE5871B-0526-4FC4-B9A6-F4984A72D176}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{154D9996-CCEC-44A4-92FD-789A7610E502}">
+          <x14:cfRule type="dataBar" id="{822BE966-7648-49EA-A3BC-01A01B84DF94}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0EFD3CFD-D976-4AC2-B422-6C53A467A85B}">
+          <x14:cfRule type="dataBar" id="{9B5B630B-C2B1-4E03-9705-78BF3C53EC96}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9EB5E666-0641-4274-B41A-CD6BAAD702FF}">
+          <x14:cfRule type="dataBar" id="{E6437F2B-05FF-44EB-9232-AB98C280E5C5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{88E62804-B35E-476D-9FE2-869194458182}">
+          <x14:cfRule type="dataBar" id="{6BE5871B-0526-4FC4-B9A6-F4984A72D176}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4E209570-8B3A-4094-9BFE-F7C8E87A30C8}</x14:id>
+          <x14:id>{62AD7AA6-D5C7-42FA-99F5-E9CAE00DD1B7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{803DFF29-392D-4BD6-A963-6EF06A3A1375}</x14:id>
+          <x14:id>{68A462F0-2497-4CD6-AA8C-A5BBFFE44C23}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C67F1B23-7383-42D8-97D7-B2C0105CF592}</x14:id>
+          <x14:id>{0CB098E5-A6C2-4D35-A9B9-5CC7B6B89124}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{35A53036-9160-40FF-B779-357515D8E1D2}</x14:id>
+          <x14:id>{29B3E539-6AA0-42E0-91B5-BB3196FCE560}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4E209570-8B3A-4094-9BFE-F7C8E87A30C8}">
+          <x14:cfRule type="dataBar" id="{62AD7AA6-D5C7-42FA-99F5-E9CAE00DD1B7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{803DFF29-392D-4BD6-A963-6EF06A3A1375}">
+          <x14:cfRule type="dataBar" id="{68A462F0-2497-4CD6-AA8C-A5BBFFE44C23}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C67F1B23-7383-42D8-97D7-B2C0105CF592}">
+          <x14:cfRule type="dataBar" id="{0CB098E5-A6C2-4D35-A9B9-5CC7B6B89124}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{35A53036-9160-40FF-B779-357515D8E1D2}">
+          <x14:cfRule type="dataBar" id="{29B3E539-6AA0-42E0-91B5-BB3196FCE560}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{822BE966-7648-49EA-A3BC-01A01B84DF94}</x14:id>
+          <x14:id>{D0052388-0A5A-4139-881D-2672A9509A77}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9B5B630B-C2B1-4E03-9705-78BF3C53EC96}</x14:id>
+          <x14:id>{74DF35EC-8BBF-400A-85AB-42A084A6AC91}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E6437F2B-05FF-44EB-9232-AB98C280E5C5}</x14:id>
+          <x14:id>{8F1E1932-AC9D-4ADC-977A-79F808A4D551}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6BE5871B-0526-4FC4-B9A6-F4984A72D176}</x14:id>
+          <x14:id>{45599B8B-7B75-4614-84A0-D29CCAEBA4A8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{822BE966-7648-49EA-A3BC-01A01B84DF94}">
+          <x14:cfRule type="dataBar" id="{D0052388-0A5A-4139-881D-2672A9509A77}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9B5B630B-C2B1-4E03-9705-78BF3C53EC96}">
+          <x14:cfRule type="dataBar" id="{74DF35EC-8BBF-400A-85AB-42A084A6AC91}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E6437F2B-05FF-44EB-9232-AB98C280E5C5}">
+          <x14:cfRule type="dataBar" id="{8F1E1932-AC9D-4ADC-977A-79F808A4D551}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6BE5871B-0526-4FC4-B9A6-F4984A72D176}">
+          <x14:cfRule type="dataBar" id="{45599B8B-7B75-4614-84A0-D29CCAEBA4A8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{62AD7AA6-D5C7-42FA-99F5-E9CAE00DD1B7}</x14:id>
+          <x14:id>{D32CDDBD-6B19-4C0D-8222-56839DD7972D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{68A462F0-2497-4CD6-AA8C-A5BBFFE44C23}</x14:id>
+          <x14:id>{A0F15126-2A46-4928-9CBB-BFA206859489}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0CB098E5-A6C2-4D35-A9B9-5CC7B6B89124}</x14:id>
+          <x14:id>{2DFC6DB7-D77D-4079-83F4-06DF0BB498D0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{29B3E539-6AA0-42E0-91B5-BB3196FCE560}</x14:id>
+          <x14:id>{5C34AC14-4ED5-48C0-9136-FF454532F20E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{62AD7AA6-D5C7-42FA-99F5-E9CAE00DD1B7}">
+          <x14:cfRule type="dataBar" id="{D32CDDBD-6B19-4C0D-8222-56839DD7972D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{68A462F0-2497-4CD6-AA8C-A5BBFFE44C23}">
+          <x14:cfRule type="dataBar" id="{A0F15126-2A46-4928-9CBB-BFA206859489}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0CB098E5-A6C2-4D35-A9B9-5CC7B6B89124}">
+          <x14:cfRule type="dataBar" id="{2DFC6DB7-D77D-4079-83F4-06DF0BB498D0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{29B3E539-6AA0-42E0-91B5-BB3196FCE560}">
+          <x14:cfRule type="dataBar" id="{5C34AC14-4ED5-48C0-9136-FF454532F20E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D0052388-0A5A-4139-881D-2672A9509A77}</x14:id>
+          <x14:id>{6F028317-5B67-4247-9582-6A7BEE31D329}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{74DF35EC-8BBF-400A-85AB-42A084A6AC91}</x14:id>
+          <x14:id>{1238320A-EAA1-4370-9DB0-5F234EED8941}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8F1E1932-AC9D-4ADC-977A-79F808A4D551}</x14:id>
+          <x14:id>{A93DD5BB-19D7-4331-A941-B8B5DD35A3B2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{45599B8B-7B75-4614-84A0-D29CCAEBA4A8}</x14:id>
+          <x14:id>{3A3886B2-A10E-4030-83B7-D8FEDEAE65D0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D0052388-0A5A-4139-881D-2672A9509A77}">
+          <x14:cfRule type="dataBar" id="{6F028317-5B67-4247-9582-6A7BEE31D329}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{74DF35EC-8BBF-400A-85AB-42A084A6AC91}">
+          <x14:cfRule type="dataBar" id="{1238320A-EAA1-4370-9DB0-5F234EED8941}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8F1E1932-AC9D-4ADC-977A-79F808A4D551}">
+          <x14:cfRule type="dataBar" id="{A93DD5BB-19D7-4331-A941-B8B5DD35A3B2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{45599B8B-7B75-4614-84A0-D29CCAEBA4A8}">
+          <x14:cfRule type="dataBar" id="{3A3886B2-A10E-4030-83B7-D8FEDEAE65D0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D32CDDBD-6B19-4C0D-8222-56839DD7972D}</x14:id>
+          <x14:id>{6D60FD2C-A98D-404F-883F-2C8A952FABFF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A0F15126-2A46-4928-9CBB-BFA206859489}</x14:id>
+          <x14:id>{5A2FE297-DE25-4AB7-8F40-6B2096609D41}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2DFC6DB7-D77D-4079-83F4-06DF0BB498D0}</x14:id>
+          <x14:id>{FD0839F0-4A47-413B-A1DA-E85C8BEAB1A0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5C34AC14-4ED5-48C0-9136-FF454532F20E}</x14:id>
+          <x14:id>{6B49BBC6-090B-4B7E-87C2-1EA9F29E3042}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D32CDDBD-6B19-4C0D-8222-56839DD7972D}">
+          <x14:cfRule type="dataBar" id="{6D60FD2C-A98D-404F-883F-2C8A952FABFF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A0F15126-2A46-4928-9CBB-BFA206859489}">
+          <x14:cfRule type="dataBar" id="{5A2FE297-DE25-4AB7-8F40-6B2096609D41}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2DFC6DB7-D77D-4079-83F4-06DF0BB498D0}">
+          <x14:cfRule type="dataBar" id="{FD0839F0-4A47-413B-A1DA-E85C8BEAB1A0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5C34AC14-4ED5-48C0-9136-FF454532F20E}">
+          <x14:cfRule type="dataBar" id="{6B49BBC6-090B-4B7E-87C2-1EA9F29E3042}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6F028317-5B67-4247-9582-6A7BEE31D329}</x14:id>
+          <x14:id>{316BFAA2-5BFB-4C7E-97C9-1A668562175F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1238320A-EAA1-4370-9DB0-5F234EED8941}</x14:id>
+          <x14:id>{B3BB1D74-FABC-48E8-920E-8CFCC9324BDE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A93DD5BB-19D7-4331-A941-B8B5DD35A3B2}</x14:id>
+          <x14:id>{28BE7FB5-C336-4262-BB7C-0CC8580CBF7D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3A3886B2-A10E-4030-83B7-D8FEDEAE65D0}</x14:id>
+          <x14:id>{E0C8D7A7-03AB-44A2-8CB4-B7CD08AEADDA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6F028317-5B67-4247-9582-6A7BEE31D329}">
+          <x14:cfRule type="dataBar" id="{316BFAA2-5BFB-4C7E-97C9-1A668562175F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1238320A-EAA1-4370-9DB0-5F234EED8941}">
+          <x14:cfRule type="dataBar" id="{B3BB1D74-FABC-48E8-920E-8CFCC9324BDE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A93DD5BB-19D7-4331-A941-B8B5DD35A3B2}">
+          <x14:cfRule type="dataBar" id="{28BE7FB5-C336-4262-BB7C-0CC8580CBF7D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3A3886B2-A10E-4030-83B7-D8FEDEAE65D0}">
+          <x14:cfRule type="dataBar" id="{E0C8D7A7-03AB-44A2-8CB4-B7CD08AEADDA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6D60FD2C-A98D-404F-883F-2C8A952FABFF}</x14:id>
+          <x14:id>{28FEFF21-57D3-4292-BB75-1068A98AE11A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5A2FE297-DE25-4AB7-8F40-6B2096609D41}</x14:id>
+          <x14:id>{4C306CF9-BF19-4B51-B52F-ABA2CC6FF479}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FD0839F0-4A47-413B-A1DA-E85C8BEAB1A0}</x14:id>
+          <x14:id>{AA2153EE-B04E-41D3-981C-4C2DDB23F4D6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6B49BBC6-090B-4B7E-87C2-1EA9F29E3042}</x14:id>
+          <x14:id>{89B6BF5E-8199-4CA4-8957-EB1BF0C02D2A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6D60FD2C-A98D-404F-883F-2C8A952FABFF}">
+          <x14:cfRule type="dataBar" id="{28FEFF21-57D3-4292-BB75-1068A98AE11A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5A2FE297-DE25-4AB7-8F40-6B2096609D41}">
+          <x14:cfRule type="dataBar" id="{4C306CF9-BF19-4B51-B52F-ABA2CC6FF479}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FD0839F0-4A47-413B-A1DA-E85C8BEAB1A0}">
+          <x14:cfRule type="dataBar" id="{AA2153EE-B04E-41D3-981C-4C2DDB23F4D6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6B49BBC6-090B-4B7E-87C2-1EA9F29E3042}">
+          <x14:cfRule type="dataBar" id="{89B6BF5E-8199-4CA4-8957-EB1BF0C02D2A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{316BFAA2-5BFB-4C7E-97C9-1A668562175F}</x14:id>
+          <x14:id>{91F9E715-9701-47A7-B81E-C5328617AF70}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B3BB1D74-FABC-48E8-920E-8CFCC9324BDE}</x14:id>
+          <x14:id>{BC626474-F0BB-40FB-8D6F-4538AD66D558}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{28BE7FB5-C336-4262-BB7C-0CC8580CBF7D}</x14:id>
+          <x14:id>{08F390F1-94B3-4E30-B3C2-49894A2F5E9A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E0C8D7A7-03AB-44A2-8CB4-B7CD08AEADDA}</x14:id>
+          <x14:id>{AB8AE95C-55F8-4593-9413-C7A7376AA78E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{316BFAA2-5BFB-4C7E-97C9-1A668562175F}">
+          <x14:cfRule type="dataBar" id="{91F9E715-9701-47A7-B81E-C5328617AF70}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B3BB1D74-FABC-48E8-920E-8CFCC9324BDE}">
+          <x14:cfRule type="dataBar" id="{BC626474-F0BB-40FB-8D6F-4538AD66D558}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{28BE7FB5-C336-4262-BB7C-0CC8580CBF7D}">
+          <x14:cfRule type="dataBar" id="{08F390F1-94B3-4E30-B3C2-49894A2F5E9A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E0C8D7A7-03AB-44A2-8CB4-B7CD08AEADDA}">
+          <x14:cfRule type="dataBar" id="{AB8AE95C-55F8-4593-9413-C7A7376AA78E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{28FEFF21-57D3-4292-BB75-1068A98AE11A}</x14:id>
+          <x14:id>{050CBC2C-DD52-4CBD-A2AF-34B46339BFA2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4C306CF9-BF19-4B51-B52F-ABA2CC6FF479}</x14:id>
+          <x14:id>{11D66CFA-725C-4156-A895-5DA54B4887B6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AA2153EE-B04E-41D3-981C-4C2DDB23F4D6}</x14:id>
+          <x14:id>{4958C96B-EDFA-41F4-B054-B54969B5BE63}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{89B6BF5E-8199-4CA4-8957-EB1BF0C02D2A}</x14:id>
+          <x14:id>{82A4C48A-761A-4B8E-80CC-93FA928FB249}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{28FEFF21-57D3-4292-BB75-1068A98AE11A}">
+          <x14:cfRule type="dataBar" id="{050CBC2C-DD52-4CBD-A2AF-34B46339BFA2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4C306CF9-BF19-4B51-B52F-ABA2CC6FF479}">
+          <x14:cfRule type="dataBar" id="{11D66CFA-725C-4156-A895-5DA54B4887B6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AA2153EE-B04E-41D3-981C-4C2DDB23F4D6}">
+          <x14:cfRule type="dataBar" id="{4958C96B-EDFA-41F4-B054-B54969B5BE63}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{89B6BF5E-8199-4CA4-8957-EB1BF0C02D2A}">
+          <x14:cfRule type="dataBar" id="{82A4C48A-761A-4B8E-80CC-93FA928FB249}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{91F9E715-9701-47A7-B81E-C5328617AF70}</x14:id>
+          <x14:id>{F59A2967-BF46-495E-99EA-5D2CDE2C751C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BC626474-F0BB-40FB-8D6F-4538AD66D558}</x14:id>
+          <x14:id>{89443C83-EFEA-47B4-8DCD-D48B926DAC5D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{08F390F1-94B3-4E30-B3C2-49894A2F5E9A}</x14:id>
+          <x14:id>{8B47587B-8637-4DB4-B32C-BF2A6563AB89}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AB8AE95C-55F8-4593-9413-C7A7376AA78E}</x14:id>
+          <x14:id>{05B0F9A5-1E4F-4877-904D-3154F8EAF102}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{91F9E715-9701-47A7-B81E-C5328617AF70}">
+          <x14:cfRule type="dataBar" id="{F59A2967-BF46-495E-99EA-5D2CDE2C751C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BC626474-F0BB-40FB-8D6F-4538AD66D558}">
+          <x14:cfRule type="dataBar" id="{89443C83-EFEA-47B4-8DCD-D48B926DAC5D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{08F390F1-94B3-4E30-B3C2-49894A2F5E9A}">
+          <x14:cfRule type="dataBar" id="{8B47587B-8637-4DB4-B32C-BF2A6563AB89}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AB8AE95C-55F8-4593-9413-C7A7376AA78E}">
+          <x14:cfRule type="dataBar" id="{05B0F9A5-1E4F-4877-904D-3154F8EAF102}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{050CBC2C-DD52-4CBD-A2AF-34B46339BFA2}</x14:id>
+          <x14:id>{96FC0B99-7B41-483E-9DDD-E62A9558557E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{11D66CFA-725C-4156-A895-5DA54B4887B6}</x14:id>
+          <x14:id>{DD4681A2-8566-45CB-897F-D0427F5B312B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4958C96B-EDFA-41F4-B054-B54969B5BE63}</x14:id>
+          <x14:id>{1286C636-816E-47D2-8A65-3E4F2B7E0534}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{82A4C48A-761A-4B8E-80CC-93FA928FB249}</x14:id>
+          <x14:id>{ECAE1195-96D7-4AB9-AC89-8DBD9EA493FA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{050CBC2C-DD52-4CBD-A2AF-34B46339BFA2}">
+          <x14:cfRule type="dataBar" id="{96FC0B99-7B41-483E-9DDD-E62A9558557E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{11D66CFA-725C-4156-A895-5DA54B4887B6}">
+          <x14:cfRule type="dataBar" id="{DD4681A2-8566-45CB-897F-D0427F5B312B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4958C96B-EDFA-41F4-B054-B54969B5BE63}">
+          <x14:cfRule type="dataBar" id="{1286C636-816E-47D2-8A65-3E4F2B7E0534}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{82A4C48A-761A-4B8E-80CC-93FA928FB249}">
+          <x14:cfRule type="dataBar" id="{ECAE1195-96D7-4AB9-AC89-8DBD9EA493FA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F59A2967-BF46-495E-99EA-5D2CDE2C751C}</x14:id>
+          <x14:id>{6E58B533-313C-4E0A-AAEE-973C4CA80450}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{89443C83-EFEA-47B4-8DCD-D48B926DAC5D}</x14:id>
+          <x14:id>{03992C93-D65A-4080-8284-81486D2D57C8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8B47587B-8637-4DB4-B32C-BF2A6563AB89}</x14:id>
+          <x14:id>{27E85237-5F08-407E-8C61-4F2D933BB2E2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{05B0F9A5-1E4F-4877-904D-3154F8EAF102}</x14:id>
+          <x14:id>{6F10E0FB-AF42-42D5-8913-2BE9AE75634E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F59A2967-BF46-495E-99EA-5D2CDE2C751C}">
+          <x14:cfRule type="dataBar" id="{6E58B533-313C-4E0A-AAEE-973C4CA80450}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{89443C83-EFEA-47B4-8DCD-D48B926DAC5D}">
+          <x14:cfRule type="dataBar" id="{03992C93-D65A-4080-8284-81486D2D57C8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8B47587B-8637-4DB4-B32C-BF2A6563AB89}">
+          <x14:cfRule type="dataBar" id="{27E85237-5F08-407E-8C61-4F2D933BB2E2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{05B0F9A5-1E4F-4877-904D-3154F8EAF102}">
+          <x14:cfRule type="dataBar" id="{6F10E0FB-AF42-42D5-8913-2BE9AE75634E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{96FC0B99-7B41-483E-9DDD-E62A9558557E}</x14:id>
+          <x14:id>{69CCE4CB-1781-4C90-A247-56D1550AFB8B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DD4681A2-8566-45CB-897F-D0427F5B312B}</x14:id>
+          <x14:id>{889369E8-8F32-4AD9-90DD-800BAA092F6D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1286C636-816E-47D2-8A65-3E4F2B7E0534}</x14:id>
+          <x14:id>{B293B7FE-1DAF-407A-B89B-480D0468E4AE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ECAE1195-96D7-4AB9-AC89-8DBD9EA493FA}</x14:id>
+          <x14:id>{117E3562-A019-4CE7-8B86-9B2836811563}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{96FC0B99-7B41-483E-9DDD-E62A9558557E}">
+          <x14:cfRule type="dataBar" id="{69CCE4CB-1781-4C90-A247-56D1550AFB8B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DD4681A2-8566-45CB-897F-D0427F5B312B}">
+          <x14:cfRule type="dataBar" id="{889369E8-8F32-4AD9-90DD-800BAA092F6D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1286C636-816E-47D2-8A65-3E4F2B7E0534}">
+          <x14:cfRule type="dataBar" id="{B293B7FE-1DAF-407A-B89B-480D0468E4AE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ECAE1195-96D7-4AB9-AC89-8DBD9EA493FA}">
+          <x14:cfRule type="dataBar" id="{117E3562-A019-4CE7-8B86-9B2836811563}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6E58B533-313C-4E0A-AAEE-973C4CA80450}</x14:id>
+          <x14:id>{F4A6A65B-183D-4413-8D07-935B3B779B50}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{03992C93-D65A-4080-8284-81486D2D57C8}</x14:id>
+          <x14:id>{8A657000-99FB-43A8-834B-D0BE9F238E96}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{27E85237-5F08-407E-8C61-4F2D933BB2E2}</x14:id>
+          <x14:id>{27676503-5DBC-4ED3-8F92-63421C89AB6F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6F10E0FB-AF42-42D5-8913-2BE9AE75634E}</x14:id>
+          <x14:id>{5EE7147D-CB01-4A4F-B205-2B2F653D4BF1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6E58B533-313C-4E0A-AAEE-973C4CA80450}">
+          <x14:cfRule type="dataBar" id="{F4A6A65B-183D-4413-8D07-935B3B779B50}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{03992C93-D65A-4080-8284-81486D2D57C8}">
+          <x14:cfRule type="dataBar" id="{8A657000-99FB-43A8-834B-D0BE9F238E96}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{27E85237-5F08-407E-8C61-4F2D933BB2E2}">
+          <x14:cfRule type="dataBar" id="{27676503-5DBC-4ED3-8F92-63421C89AB6F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6F10E0FB-AF42-42D5-8913-2BE9AE75634E}">
+          <x14:cfRule type="dataBar" id="{5EE7147D-CB01-4A4F-B205-2B2F653D4BF1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{69CCE4CB-1781-4C90-A247-56D1550AFB8B}</x14:id>
+          <x14:id>{EEE7BE54-6F31-4A29-8EC5-99AE45827B08}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{889369E8-8F32-4AD9-90DD-800BAA092F6D}</x14:id>
+          <x14:id>{E51E1FBB-D685-4392-BF0A-9CC4365BAE5A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B293B7FE-1DAF-407A-B89B-480D0468E4AE}</x14:id>
+          <x14:id>{CD87E968-9238-4201-92D8-4EB88FE04A3D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{117E3562-A019-4CE7-8B86-9B2836811563}</x14:id>
+          <x14:id>{716D2F56-DE42-46DC-BA03-9F5A7DD7C829}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{69CCE4CB-1781-4C90-A247-56D1550AFB8B}">
+          <x14:cfRule type="dataBar" id="{EEE7BE54-6F31-4A29-8EC5-99AE45827B08}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{889369E8-8F32-4AD9-90DD-800BAA092F6D}">
+          <x14:cfRule type="dataBar" id="{E51E1FBB-D685-4392-BF0A-9CC4365BAE5A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B293B7FE-1DAF-407A-B89B-480D0468E4AE}">
+          <x14:cfRule type="dataBar" id="{CD87E968-9238-4201-92D8-4EB88FE04A3D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{117E3562-A019-4CE7-8B86-9B2836811563}">
+          <x14:cfRule type="dataBar" id="{716D2F56-DE42-46DC-BA03-9F5A7DD7C829}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F4A6A65B-183D-4413-8D07-935B3B779B50}</x14:id>
+          <x14:id>{60794FB7-8BB4-4C4B-8055-18209C38DBDE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8A657000-99FB-43A8-834B-D0BE9F238E96}</x14:id>
+          <x14:id>{356DEEFE-EE5F-42E3-B03D-824678A775A9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{27676503-5DBC-4ED3-8F92-63421C89AB6F}</x14:id>
+          <x14:id>{555AE085-6FEA-47C3-A241-156BE08F78AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5EE7147D-CB01-4A4F-B205-2B2F653D4BF1}</x14:id>
+          <x14:id>{AAD50BD9-3206-4214-B709-086A2ECBE3D1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F4A6A65B-183D-4413-8D07-935B3B779B50}">
+          <x14:cfRule type="dataBar" id="{60794FB7-8BB4-4C4B-8055-18209C38DBDE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8A657000-99FB-43A8-834B-D0BE9F238E96}">
+          <x14:cfRule type="dataBar" id="{356DEEFE-EE5F-42E3-B03D-824678A775A9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{27676503-5DBC-4ED3-8F92-63421C89AB6F}">
+          <x14:cfRule type="dataBar" id="{555AE085-6FEA-47C3-A241-156BE08F78AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5EE7147D-CB01-4A4F-B205-2B2F653D4BF1}">
+          <x14:cfRule type="dataBar" id="{AAD50BD9-3206-4214-B709-086A2ECBE3D1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 08:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EEE7BE54-6F31-4A29-8EC5-99AE45827B08}</x14:id>
+          <x14:id>{70200E08-C27C-4010-8DA5-E68A708B03FF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E51E1FBB-D685-4392-BF0A-9CC4365BAE5A}</x14:id>
+          <x14:id>{DF9EBC0B-B461-45F5-A7CF-232F4BD0E811}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CD87E968-9238-4201-92D8-4EB88FE04A3D}</x14:id>
+          <x14:id>{AF177E1B-CCC1-4F05-B568-5C59C66CEDE5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{716D2F56-DE42-46DC-BA03-9F5A7DD7C829}</x14:id>
+          <x14:id>{47AB4B21-B830-4427-9F51-79EF5975801F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EEE7BE54-6F31-4A29-8EC5-99AE45827B08}">
+          <x14:cfRule type="dataBar" id="{70200E08-C27C-4010-8DA5-E68A708B03FF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E51E1FBB-D685-4392-BF0A-9CC4365BAE5A}">
+          <x14:cfRule type="dataBar" id="{DF9EBC0B-B461-45F5-A7CF-232F4BD0E811}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CD87E968-9238-4201-92D8-4EB88FE04A3D}">
+          <x14:cfRule type="dataBar" id="{AF177E1B-CCC1-4F05-B568-5C59C66CEDE5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{716D2F56-DE42-46DC-BA03-9F5A7DD7C829}">
+          <x14:cfRule type="dataBar" id="{47AB4B21-B830-4427-9F51-79EF5975801F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{60794FB7-8BB4-4C4B-8055-18209C38DBDE}</x14:id>
+          <x14:id>{0481E612-70E4-40D3-9F84-F7706B9A7C3A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{356DEEFE-EE5F-42E3-B03D-824678A775A9}</x14:id>
+          <x14:id>{A7EE08CC-EE0C-4B9A-9E42-E2C179D50F92}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{555AE085-6FEA-47C3-A241-156BE08F78AB}</x14:id>
+          <x14:id>{EE297706-3430-416F-9AC0-8719C80AE416}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AAD50BD9-3206-4214-B709-086A2ECBE3D1}</x14:id>
+          <x14:id>{DC0D3955-2E44-42D4-B735-AD07A50730B7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{60794FB7-8BB4-4C4B-8055-18209C38DBDE}">
+          <x14:cfRule type="dataBar" id="{0481E612-70E4-40D3-9F84-F7706B9A7C3A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{356DEEFE-EE5F-42E3-B03D-824678A775A9}">
+          <x14:cfRule type="dataBar" id="{A7EE08CC-EE0C-4B9A-9E42-E2C179D50F92}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{555AE085-6FEA-47C3-A241-156BE08F78AB}">
+          <x14:cfRule type="dataBar" id="{EE297706-3430-416F-9AC0-8719C80AE416}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AAD50BD9-3206-4214-B709-086A2ECBE3D1}">
+          <x14:cfRule type="dataBar" id="{DC0D3955-2E44-42D4-B735-AD07A50730B7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{70200E08-C27C-4010-8DA5-E68A708B03FF}</x14:id>
+          <x14:id>{9440386F-7E48-425B-8B03-C2441B8E824E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DF9EBC0B-B461-45F5-A7CF-232F4BD0E811}</x14:id>
+          <x14:id>{939FDCDB-D504-4D1B-9AF9-925423513EBA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AF177E1B-CCC1-4F05-B568-5C59C66CEDE5}</x14:id>
+          <x14:id>{00DED626-3FAC-446A-A148-AF4A663F319B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{47AB4B21-B830-4427-9F51-79EF5975801F}</x14:id>
+          <x14:id>{ABE63613-ABB3-4728-8857-BC4930649E2C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{70200E08-C27C-4010-8DA5-E68A708B03FF}">
+          <x14:cfRule type="dataBar" id="{9440386F-7E48-425B-8B03-C2441B8E824E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DF9EBC0B-B461-45F5-A7CF-232F4BD0E811}">
+          <x14:cfRule type="dataBar" id="{939FDCDB-D504-4D1B-9AF9-925423513EBA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AF177E1B-CCC1-4F05-B568-5C59C66CEDE5}">
+          <x14:cfRule type="dataBar" id="{00DED626-3FAC-446A-A148-AF4A663F319B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{47AB4B21-B830-4427-9F51-79EF5975801F}">
+          <x14:cfRule type="dataBar" id="{ABE63613-ABB3-4728-8857-BC4930649E2C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0481E612-70E4-40D3-9F84-F7706B9A7C3A}</x14:id>
+          <x14:id>{1EC57250-E9DD-400A-B466-EBA3804B0FDE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A7EE08CC-EE0C-4B9A-9E42-E2C179D50F92}</x14:id>
+          <x14:id>{78FA1D2A-8F2B-423E-A4BA-DFA0DEB0F888}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EE297706-3430-416F-9AC0-8719C80AE416}</x14:id>
+          <x14:id>{C183BEAF-5488-459B-B6BA-52B3251245B3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DC0D3955-2E44-42D4-B735-AD07A50730B7}</x14:id>
+          <x14:id>{E88B710F-4CCB-4589-AC32-B4BE42C7C437}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0481E612-70E4-40D3-9F84-F7706B9A7C3A}">
+          <x14:cfRule type="dataBar" id="{1EC57250-E9DD-400A-B466-EBA3804B0FDE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A7EE08CC-EE0C-4B9A-9E42-E2C179D50F92}">
+          <x14:cfRule type="dataBar" id="{78FA1D2A-8F2B-423E-A4BA-DFA0DEB0F888}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EE297706-3430-416F-9AC0-8719C80AE416}">
+          <x14:cfRule type="dataBar" id="{C183BEAF-5488-459B-B6BA-52B3251245B3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DC0D3955-2E44-42D4-B735-AD07A50730B7}">
+          <x14:cfRule type="dataBar" id="{E88B710F-4CCB-4589-AC32-B4BE42C7C437}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:05Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9440386F-7E48-425B-8B03-C2441B8E824E}</x14:id>
+          <x14:id>{95C0D33C-4ED2-4E55-9C73-27D7F11F8C64}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{939FDCDB-D504-4D1B-9AF9-925423513EBA}</x14:id>
+          <x14:id>{0C019577-9E67-4B19-AB96-707835F0D313}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{00DED626-3FAC-446A-A148-AF4A663F319B}</x14:id>
+          <x14:id>{53CF6419-9A06-44A5-BA45-461F81240951}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ABE63613-ABB3-4728-8857-BC4930649E2C}</x14:id>
+          <x14:id>{26E40D35-A91A-4FD5-AAD7-CD753ACB208F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9440386F-7E48-425B-8B03-C2441B8E824E}">
+          <x14:cfRule type="dataBar" id="{95C0D33C-4ED2-4E55-9C73-27D7F11F8C64}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{939FDCDB-D504-4D1B-9AF9-925423513EBA}">
+          <x14:cfRule type="dataBar" id="{0C019577-9E67-4B19-AB96-707835F0D313}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{00DED626-3FAC-446A-A148-AF4A663F319B}">
+          <x14:cfRule type="dataBar" id="{53CF6419-9A06-44A5-BA45-461F81240951}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ABE63613-ABB3-4728-8857-BC4930649E2C}">
+          <x14:cfRule type="dataBar" id="{26E40D35-A91A-4FD5-AAD7-CD753ACB208F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1EC57250-E9DD-400A-B466-EBA3804B0FDE}</x14:id>
+          <x14:id>{FCF3C963-E2D1-4209-B51A-C798D165EBD6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{78FA1D2A-8F2B-423E-A4BA-DFA0DEB0F888}</x14:id>
+          <x14:id>{F53D686D-394C-4165-8540-2E1D0A7B7856}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C183BEAF-5488-459B-B6BA-52B3251245B3}</x14:id>
+          <x14:id>{DB9E9DCA-17BD-47B6-9529-14DBA02D4E6D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E88B710F-4CCB-4589-AC32-B4BE42C7C437}</x14:id>
+          <x14:id>{242B28B3-BFB3-4834-9E29-4C4D1E85725E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1EC57250-E9DD-400A-B466-EBA3804B0FDE}">
+          <x14:cfRule type="dataBar" id="{FCF3C963-E2D1-4209-B51A-C798D165EBD6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{78FA1D2A-8F2B-423E-A4BA-DFA0DEB0F888}">
+          <x14:cfRule type="dataBar" id="{F53D686D-394C-4165-8540-2E1D0A7B7856}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C183BEAF-5488-459B-B6BA-52B3251245B3}">
+          <x14:cfRule type="dataBar" id="{DB9E9DCA-17BD-47B6-9529-14DBA02D4E6D}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E88B710F-4CCB-4589-AC32-B4BE42C7C437}">
+          <x14:cfRule type="dataBar" id="{242B28B3-BFB3-4834-9E29-4C4D1E85725E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:10Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{95C0D33C-4ED2-4E55-9C73-27D7F11F8C64}</x14:id>
+          <x14:id>{49952A7C-7722-4B2F-B6FD-4E9E079CB78A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0C019577-9E67-4B19-AB96-707835F0D313}</x14:id>
+          <x14:id>{58DB5380-C9F6-42E6-8F4E-87479D584A5B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{53CF6419-9A06-44A5-BA45-461F81240951}</x14:id>
+          <x14:id>{05C18CAD-C6FE-476A-B70E-752A546826D5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{26E40D35-A91A-4FD5-AAD7-CD753ACB208F}</x14:id>
+          <x14:id>{FC532576-53E5-411E-B1D2-32CB0632E8A3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{95C0D33C-4ED2-4E55-9C73-27D7F11F8C64}">
+          <x14:cfRule type="dataBar" id="{49952A7C-7722-4B2F-B6FD-4E9E079CB78A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0C019577-9E67-4B19-AB96-707835F0D313}">
+          <x14:cfRule type="dataBar" id="{58DB5380-C9F6-42E6-8F4E-87479D584A5B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{53CF6419-9A06-44A5-BA45-461F81240951}">
+          <x14:cfRule type="dataBar" id="{05C18CAD-C6FE-476A-B70E-752A546826D5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{26E40D35-A91A-4FD5-AAD7-CD753ACB208F}">
+          <x14:cfRule type="dataBar" id="{FC532576-53E5-411E-B1D2-32CB0632E8A3}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FCF3C963-E2D1-4209-B51A-C798D165EBD6}</x14:id>
+          <x14:id>{67701479-0BFB-46E3-82A4-18C732DE43A4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F53D686D-394C-4165-8540-2E1D0A7B7856}</x14:id>
+          <x14:id>{E5547AFC-62BA-48D4-A5BD-DAEC35EBF3B7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DB9E9DCA-17BD-47B6-9529-14DBA02D4E6D}</x14:id>
+          <x14:id>{A3A60072-E435-4498-BDFA-AACF9EF19055}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{242B28B3-BFB3-4834-9E29-4C4D1E85725E}</x14:id>
+          <x14:id>{79A1DBCA-698A-43C6-9E6F-459084566803}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FCF3C963-E2D1-4209-B51A-C798D165EBD6}">
+          <x14:cfRule type="dataBar" id="{67701479-0BFB-46E3-82A4-18C732DE43A4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F53D686D-394C-4165-8540-2E1D0A7B7856}">
+          <x14:cfRule type="dataBar" id="{E5547AFC-62BA-48D4-A5BD-DAEC35EBF3B7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DB9E9DCA-17BD-47B6-9529-14DBA02D4E6D}">
+          <x14:cfRule type="dataBar" id="{A3A60072-E435-4498-BDFA-AACF9EF19055}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{242B28B3-BFB3-4834-9E29-4C4D1E85725E}">
+          <x14:cfRule type="dataBar" id="{79A1DBCA-698A-43C6-9E6F-459084566803}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{49952A7C-7722-4B2F-B6FD-4E9E079CB78A}</x14:id>
+          <x14:id>{2A5C0846-EF58-4D73-B7D9-0C7B89F878E6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{58DB5380-C9F6-42E6-8F4E-87479D584A5B}</x14:id>
+          <x14:id>{FAB18A47-0FE0-4978-B578-1835F6E0D075}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{05C18CAD-C6FE-476A-B70E-752A546826D5}</x14:id>
+          <x14:id>{2EEB438B-827D-4725-B23E-EA78613316F2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FC532576-53E5-411E-B1D2-32CB0632E8A3}</x14:id>
+          <x14:id>{45514427-2952-4015-B0F0-F29AB7A75C66}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{49952A7C-7722-4B2F-B6FD-4E9E079CB78A}">
+          <x14:cfRule type="dataBar" id="{2A5C0846-EF58-4D73-B7D9-0C7B89F878E6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{58DB5380-C9F6-42E6-8F4E-87479D584A5B}">
+          <x14:cfRule type="dataBar" id="{FAB18A47-0FE0-4978-B578-1835F6E0D075}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{05C18CAD-C6FE-476A-B70E-752A546826D5}">
+          <x14:cfRule type="dataBar" id="{2EEB438B-827D-4725-B23E-EA78613316F2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FC532576-53E5-411E-B1D2-32CB0632E8A3}">
+          <x14:cfRule type="dataBar" id="{45514427-2952-4015-B0F0-F29AB7A75C66}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{67701479-0BFB-46E3-82A4-18C732DE43A4}</x14:id>
+          <x14:id>{E57B226D-701A-47F7-B4DB-3BFCF1026D37}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E5547AFC-62BA-48D4-A5BD-DAEC35EBF3B7}</x14:id>
+          <x14:id>{434D5F1F-4D5B-4D45-AB79-ABAC49F0367A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A3A60072-E435-4498-BDFA-AACF9EF19055}</x14:id>
+          <x14:id>{A6D27B5B-57A0-4B3D-BD0D-952571B83F28}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{79A1DBCA-698A-43C6-9E6F-459084566803}</x14:id>
+          <x14:id>{88EA59EA-D8E8-44B8-B705-A6368C5A6AFD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{67701479-0BFB-46E3-82A4-18C732DE43A4}">
+          <x14:cfRule type="dataBar" id="{E57B226D-701A-47F7-B4DB-3BFCF1026D37}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E5547AFC-62BA-48D4-A5BD-DAEC35EBF3B7}">
+          <x14:cfRule type="dataBar" id="{434D5F1F-4D5B-4D45-AB79-ABAC49F0367A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A3A60072-E435-4498-BDFA-AACF9EF19055}">
+          <x14:cfRule type="dataBar" id="{A6D27B5B-57A0-4B3D-BD0D-952571B83F28}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{79A1DBCA-698A-43C6-9E6F-459084566803}">
+          <x14:cfRule type="dataBar" id="{88EA59EA-D8E8-44B8-B705-A6368C5A6AFD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:20Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2A5C0846-EF58-4D73-B7D9-0C7B89F878E6}</x14:id>
+          <x14:id>{3063C548-7ECE-4F99-A9D3-7F9312B4F987}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FAB18A47-0FE0-4978-B578-1835F6E0D075}</x14:id>
+          <x14:id>{90B2010B-E28A-45A8-A25A-F661A19BB4AC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2EEB438B-827D-4725-B23E-EA78613316F2}</x14:id>
+          <x14:id>{26910F71-ABDA-4187-9339-53BBABD60B2A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{45514427-2952-4015-B0F0-F29AB7A75C66}</x14:id>
+          <x14:id>{77569140-C148-49A4-ADB6-B2373188F002}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2A5C0846-EF58-4D73-B7D9-0C7B89F878E6}">
+          <x14:cfRule type="dataBar" id="{3063C548-7ECE-4F99-A9D3-7F9312B4F987}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FAB18A47-0FE0-4978-B578-1835F6E0D075}">
+          <x14:cfRule type="dataBar" id="{90B2010B-E28A-45A8-A25A-F661A19BB4AC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2EEB438B-827D-4725-B23E-EA78613316F2}">
+          <x14:cfRule type="dataBar" id="{26910F71-ABDA-4187-9339-53BBABD60B2A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{45514427-2952-4015-B0F0-F29AB7A75C66}">
+          <x14:cfRule type="dataBar" id="{77569140-C148-49A4-ADB6-B2373188F002}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E57B226D-701A-47F7-B4DB-3BFCF1026D37}</x14:id>
+          <x14:id>{7D56C63C-E43D-4E32-9C29-3AA0C5A301E9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{434D5F1F-4D5B-4D45-AB79-ABAC49F0367A}</x14:id>
+          <x14:id>{32C4761B-EA45-4ED6-BA31-F672006BF8D4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A6D27B5B-57A0-4B3D-BD0D-952571B83F28}</x14:id>
+          <x14:id>{CFC0FC5E-83B3-40A5-875B-AD9819202ECA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{88EA59EA-D8E8-44B8-B705-A6368C5A6AFD}</x14:id>
+          <x14:id>{D75EF744-BFCE-4155-A117-B5F850CF770A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E57B226D-701A-47F7-B4DB-3BFCF1026D37}">
+          <x14:cfRule type="dataBar" id="{7D56C63C-E43D-4E32-9C29-3AA0C5A301E9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{434D5F1F-4D5B-4D45-AB79-ABAC49F0367A}">
+          <x14:cfRule type="dataBar" id="{32C4761B-EA45-4ED6-BA31-F672006BF8D4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A6D27B5B-57A0-4B3D-BD0D-952571B83F28}">
+          <x14:cfRule type="dataBar" id="{CFC0FC5E-83B3-40A5-875B-AD9819202ECA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{88EA59EA-D8E8-44B8-B705-A6368C5A6AFD}">
+          <x14:cfRule type="dataBar" id="{D75EF744-BFCE-4155-A117-B5F850CF770A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:25Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3063C548-7ECE-4F99-A9D3-7F9312B4F987}</x14:id>
+          <x14:id>{79BBA9A6-A756-4B6E-BF60-E4BDC84CD43A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{90B2010B-E28A-45A8-A25A-F661A19BB4AC}</x14:id>
+          <x14:id>{FB454601-3F59-4D4D-9BCA-9F3A2E4DD082}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{26910F71-ABDA-4187-9339-53BBABD60B2A}</x14:id>
+          <x14:id>{E4BEEAF8-A1A0-4EAF-8F25-9762B395F4F1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{77569140-C148-49A4-ADB6-B2373188F002}</x14:id>
+          <x14:id>{BF593270-597F-4393-9B2A-C1F34E7244EA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3063C548-7ECE-4F99-A9D3-7F9312B4F987}">
+          <x14:cfRule type="dataBar" id="{79BBA9A6-A756-4B6E-BF60-E4BDC84CD43A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{90B2010B-E28A-45A8-A25A-F661A19BB4AC}">
+          <x14:cfRule type="dataBar" id="{FB454601-3F59-4D4D-9BCA-9F3A2E4DD082}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{26910F71-ABDA-4187-9339-53BBABD60B2A}">
+          <x14:cfRule type="dataBar" id="{E4BEEAF8-A1A0-4EAF-8F25-9762B395F4F1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{77569140-C148-49A4-ADB6-B2373188F002}">
+          <x14:cfRule type="dataBar" id="{BF593270-597F-4393-9B2A-C1F34E7244EA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7D56C63C-E43D-4E32-9C29-3AA0C5A301E9}</x14:id>
+          <x14:id>{B30A5449-C80D-4A24-8744-9B8F4D247856}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{32C4761B-EA45-4ED6-BA31-F672006BF8D4}</x14:id>
+          <x14:id>{32011F19-BD89-4A91-A813-9FBBE9FFBBEB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CFC0FC5E-83B3-40A5-875B-AD9819202ECA}</x14:id>
+          <x14:id>{5605E363-5595-4B59-B41E-09C8792E949C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D75EF744-BFCE-4155-A117-B5F850CF770A}</x14:id>
+          <x14:id>{13E52AD9-782C-4343-BBC7-28600C179A16}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7D56C63C-E43D-4E32-9C29-3AA0C5A301E9}">
+          <x14:cfRule type="dataBar" id="{B30A5449-C80D-4A24-8744-9B8F4D247856}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{32C4761B-EA45-4ED6-BA31-F672006BF8D4}">
+          <x14:cfRule type="dataBar" id="{32011F19-BD89-4A91-A813-9FBBE9FFBBEB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CFC0FC5E-83B3-40A5-875B-AD9819202ECA}">
+          <x14:cfRule type="dataBar" id="{5605E363-5595-4B59-B41E-09C8792E949C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D75EF744-BFCE-4155-A117-B5F850CF770A}">
+          <x14:cfRule type="dataBar" id="{13E52AD9-782C-4343-BBC7-28600C179A16}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:30Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{79BBA9A6-A756-4B6E-BF60-E4BDC84CD43A}</x14:id>
+          <x14:id>{A1404A41-97AD-4DC9-B3DD-6E868808DFAE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FB454601-3F59-4D4D-9BCA-9F3A2E4DD082}</x14:id>
+          <x14:id>{2725003F-5443-450D-BF70-8ADEF64EDF92}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E4BEEAF8-A1A0-4EAF-8F25-9762B395F4F1}</x14:id>
+          <x14:id>{F45C87E1-90E8-4AD9-8289-E4525AD27B89}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BF593270-597F-4393-9B2A-C1F34E7244EA}</x14:id>
+          <x14:id>{AFD26246-F04C-4D17-9655-81E3D56BA8FD}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{79BBA9A6-A756-4B6E-BF60-E4BDC84CD43A}">
+          <x14:cfRule type="dataBar" id="{A1404A41-97AD-4DC9-B3DD-6E868808DFAE}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FB454601-3F59-4D4D-9BCA-9F3A2E4DD082}">
+          <x14:cfRule type="dataBar" id="{2725003F-5443-450D-BF70-8ADEF64EDF92}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E4BEEAF8-A1A0-4EAF-8F25-9762B395F4F1}">
+          <x14:cfRule type="dataBar" id="{F45C87E1-90E8-4AD9-8289-E4525AD27B89}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BF593270-597F-4393-9B2A-C1F34E7244EA}">
+          <x14:cfRule type="dataBar" id="{AFD26246-F04C-4D17-9655-81E3D56BA8FD}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B30A5449-C80D-4A24-8744-9B8F4D247856}</x14:id>
+          <x14:id>{BB51E152-BE3F-4469-9138-D3FBC7E86C86}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{32011F19-BD89-4A91-A813-9FBBE9FFBBEB}</x14:id>
+          <x14:id>{18F2D09D-9D21-40FE-82CB-AB394ED44F32}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5605E363-5595-4B59-B41E-09C8792E949C}</x14:id>
+          <x14:id>{0D3C5E8A-BF54-4057-83CE-8C3E8C198AA4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{13E52AD9-782C-4343-BBC7-28600C179A16}</x14:id>
+          <x14:id>{B7A163A2-337C-4CAE-A253-12F557EE3018}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B30A5449-C80D-4A24-8744-9B8F4D247856}">
+          <x14:cfRule type="dataBar" id="{BB51E152-BE3F-4469-9138-D3FBC7E86C86}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{32011F19-BD89-4A91-A813-9FBBE9FFBBEB}">
+          <x14:cfRule type="dataBar" id="{18F2D09D-9D21-40FE-82CB-AB394ED44F32}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5605E363-5595-4B59-B41E-09C8792E949C}">
+          <x14:cfRule type="dataBar" id="{0D3C5E8A-BF54-4057-83CE-8C3E8C198AA4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{13E52AD9-782C-4343-BBC7-28600C179A16}">
+          <x14:cfRule type="dataBar" id="{B7A163A2-337C-4CAE-A253-12F557EE3018}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:35Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A1404A41-97AD-4DC9-B3DD-6E868808DFAE}</x14:id>
+          <x14:id>{55EB3A8C-8588-4EB3-BF4A-CF86D4925082}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2725003F-5443-450D-BF70-8ADEF64EDF92}</x14:id>
+          <x14:id>{8CE16BE8-2CCA-4DD3-A419-7D12C81D1585}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F45C87E1-90E8-4AD9-8289-E4525AD27B89}</x14:id>
+          <x14:id>{3941B78F-6514-48D8-B79A-9E3BBE457CF8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AFD26246-F04C-4D17-9655-81E3D56BA8FD}</x14:id>
+          <x14:id>{EFCA95F0-0BA0-4916-921A-4FC137422792}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A1404A41-97AD-4DC9-B3DD-6E868808DFAE}">
+          <x14:cfRule type="dataBar" id="{55EB3A8C-8588-4EB3-BF4A-CF86D4925082}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2725003F-5443-450D-BF70-8ADEF64EDF92}">
+          <x14:cfRule type="dataBar" id="{8CE16BE8-2CCA-4DD3-A419-7D12C81D1585}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F45C87E1-90E8-4AD9-8289-E4525AD27B89}">
+          <x14:cfRule type="dataBar" id="{3941B78F-6514-48D8-B79A-9E3BBE457CF8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AFD26246-F04C-4D17-9655-81E3D56BA8FD}">
+          <x14:cfRule type="dataBar" id="{EFCA95F0-0BA0-4916-921A-4FC137422792}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BB51E152-BE3F-4469-9138-D3FBC7E86C86}</x14:id>
+          <x14:id>{A182A089-E945-461A-8A51-7E8E1386E390}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{18F2D09D-9D21-40FE-82CB-AB394ED44F32}</x14:id>
+          <x14:id>{816F5FED-0B8D-4393-B96B-C4A533857E0F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0D3C5E8A-BF54-4057-83CE-8C3E8C198AA4}</x14:id>
+          <x14:id>{E1872C55-6994-4B3C-9CC2-E8DFB61CC3DA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B7A163A2-337C-4CAE-A253-12F557EE3018}</x14:id>
+          <x14:id>{C51F75A1-4A5A-4D31-A3B7-998F397116F2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BB51E152-BE3F-4469-9138-D3FBC7E86C86}">
+          <x14:cfRule type="dataBar" id="{A182A089-E945-461A-8A51-7E8E1386E390}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{18F2D09D-9D21-40FE-82CB-AB394ED44F32}">
+          <x14:cfRule type="dataBar" id="{816F5FED-0B8D-4393-B96B-C4A533857E0F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0D3C5E8A-BF54-4057-83CE-8C3E8C198AA4}">
+          <x14:cfRule type="dataBar" id="{E1872C55-6994-4B3C-9CC2-E8DFB61CC3DA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B7A163A2-337C-4CAE-A253-12F557EE3018}">
+          <x14:cfRule type="dataBar" id="{C51F75A1-4A5A-4D31-A3B7-998F397116F2}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:40Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{55EB3A8C-8588-4EB3-BF4A-CF86D4925082}</x14:id>
+          <x14:id>{5C61D934-10A9-4921-9865-ECBAF4D5CAD1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8CE16BE8-2CCA-4DD3-A419-7D12C81D1585}</x14:id>
+          <x14:id>{A8987373-CF1C-4113-A30E-CEC664A81C87}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3941B78F-6514-48D8-B79A-9E3BBE457CF8}</x14:id>
+          <x14:id>{3A1BF486-6575-491B-97AA-EA805BF1A778}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EFCA95F0-0BA0-4916-921A-4FC137422792}</x14:id>
+          <x14:id>{E0244867-1929-4274-8224-666801E946AC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{55EB3A8C-8588-4EB3-BF4A-CF86D4925082}">
+          <x14:cfRule type="dataBar" id="{5C61D934-10A9-4921-9865-ECBAF4D5CAD1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8CE16BE8-2CCA-4DD3-A419-7D12C81D1585}">
+          <x14:cfRule type="dataBar" id="{A8987373-CF1C-4113-A30E-CEC664A81C87}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3941B78F-6514-48D8-B79A-9E3BBE457CF8}">
+          <x14:cfRule type="dataBar" id="{3A1BF486-6575-491B-97AA-EA805BF1A778}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EFCA95F0-0BA0-4916-921A-4FC137422792}">
+          <x14:cfRule type="dataBar" id="{E0244867-1929-4274-8224-666801E946AC}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A182A089-E945-461A-8A51-7E8E1386E390}</x14:id>
+          <x14:id>{202AB13C-3474-4625-AE70-4C9FACCB17E6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{816F5FED-0B8D-4393-B96B-C4A533857E0F}</x14:id>
+          <x14:id>{38BF195C-FE69-4764-A7B0-6332AA2231CB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E1872C55-6994-4B3C-9CC2-E8DFB61CC3DA}</x14:id>
+          <x14:id>{AB7B93E8-4436-4991-9F54-6C3517FC9129}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C51F75A1-4A5A-4D31-A3B7-998F397116F2}</x14:id>
+          <x14:id>{F1031250-A454-4173-968E-82D221DC656A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A182A089-E945-461A-8A51-7E8E1386E390}">
+          <x14:cfRule type="dataBar" id="{202AB13C-3474-4625-AE70-4C9FACCB17E6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{816F5FED-0B8D-4393-B96B-C4A533857E0F}">
+          <x14:cfRule type="dataBar" id="{38BF195C-FE69-4764-A7B0-6332AA2231CB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E1872C55-6994-4B3C-9CC2-E8DFB61CC3DA}">
+          <x14:cfRule type="dataBar" id="{AB7B93E8-4436-4991-9F54-6C3517FC9129}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C51F75A1-4A5A-4D31-A3B7-998F397116F2}">
+          <x14:cfRule type="dataBar" id="{F1031250-A454-4173-968E-82D221DC656A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:45Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5C61D934-10A9-4921-9865-ECBAF4D5CAD1}</x14:id>
+          <x14:id>{389D1FFA-4444-42F5-A872-FE134F9FB7A1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A8987373-CF1C-4113-A30E-CEC664A81C87}</x14:id>
+          <x14:id>{7195EF76-CE4A-49C2-ABA7-F7A2A67854E4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3A1BF486-6575-491B-97AA-EA805BF1A778}</x14:id>
+          <x14:id>{018A77E0-6FD4-40E4-BCBC-F5A5E207DF3A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E0244867-1929-4274-8224-666801E946AC}</x14:id>
+          <x14:id>{2F86BD86-FF21-47D4-B4C1-B821B2EF4D6E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5C61D934-10A9-4921-9865-ECBAF4D5CAD1}">
+          <x14:cfRule type="dataBar" id="{389D1FFA-4444-42F5-A872-FE134F9FB7A1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A8987373-CF1C-4113-A30E-CEC664A81C87}">
+          <x14:cfRule type="dataBar" id="{7195EF76-CE4A-49C2-ABA7-F7A2A67854E4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3A1BF486-6575-491B-97AA-EA805BF1A778}">
+          <x14:cfRule type="dataBar" id="{018A77E0-6FD4-40E4-BCBC-F5A5E207DF3A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E0244867-1929-4274-8224-666801E946AC}">
+          <x14:cfRule type="dataBar" id="{2F86BD86-FF21-47D4-B4C1-B821B2EF4D6E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{202AB13C-3474-4625-AE70-4C9FACCB17E6}</x14:id>
+          <x14:id>{89D2D125-82D9-46BA-AAE0-8A0D7F44A073}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{38BF195C-FE69-4764-A7B0-6332AA2231CB}</x14:id>
+          <x14:id>{8574E2C1-D780-4071-B61E-C0067B9522CF}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AB7B93E8-4436-4991-9F54-6C3517FC9129}</x14:id>
+          <x14:id>{CBBED15E-BBB3-455F-821B-A1A095CA4B6A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F1031250-A454-4173-968E-82D221DC656A}</x14:id>
+          <x14:id>{893E9808-35B4-4B23-8E3A-9E678260F4AB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{202AB13C-3474-4625-AE70-4C9FACCB17E6}">
+          <x14:cfRule type="dataBar" id="{89D2D125-82D9-46BA-AAE0-8A0D7F44A073}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{38BF195C-FE69-4764-A7B0-6332AA2231CB}">
+          <x14:cfRule type="dataBar" id="{8574E2C1-D780-4071-B61E-C0067B9522CF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AB7B93E8-4436-4991-9F54-6C3517FC9129}">
+          <x14:cfRule type="dataBar" id="{CBBED15E-BBB3-455F-821B-A1A095CA4B6A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F1031250-A454-4173-968E-82D221DC656A}">
+          <x14:cfRule type="dataBar" id="{893E9808-35B4-4B23-8E3A-9E678260F4AB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:50Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{389D1FFA-4444-42F5-A872-FE134F9FB7A1}</x14:id>
+          <x14:id>{07189A70-7105-49DC-AE0D-6C69942BF1D5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7195EF76-CE4A-49C2-ABA7-F7A2A67854E4}</x14:id>
+          <x14:id>{6C72F6D7-DE14-43D2-8115-CC2E4D0ACB7C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{018A77E0-6FD4-40E4-BCBC-F5A5E207DF3A}</x14:id>
+          <x14:id>{ECDB0782-B748-4AC1-9999-3FCD9B30DB86}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2F86BD86-FF21-47D4-B4C1-B821B2EF4D6E}</x14:id>
+          <x14:id>{E138A6EC-DEBF-4C7B-A602-99ED8F3A0C8E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{389D1FFA-4444-42F5-A872-FE134F9FB7A1}">
+          <x14:cfRule type="dataBar" id="{07189A70-7105-49DC-AE0D-6C69942BF1D5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7195EF76-CE4A-49C2-ABA7-F7A2A67854E4}">
+          <x14:cfRule type="dataBar" id="{6C72F6D7-DE14-43D2-8115-CC2E4D0ACB7C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{018A77E0-6FD4-40E4-BCBC-F5A5E207DF3A}">
+          <x14:cfRule type="dataBar" id="{ECDB0782-B748-4AC1-9999-3FCD9B30DB86}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2F86BD86-FF21-47D4-B4C1-B821B2EF4D6E}">
+          <x14:cfRule type="dataBar" id="{E138A6EC-DEBF-4C7B-A602-99ED8F3A0C8E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{89D2D125-82D9-46BA-AAE0-8A0D7F44A073}</x14:id>
+          <x14:id>{6F640BA9-0B24-4E26-A635-36AF932E75BB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8574E2C1-D780-4071-B61E-C0067B9522CF}</x14:id>
+          <x14:id>{7F9127B5-A116-465D-951E-88D3559AAFE4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CBBED15E-BBB3-455F-821B-A1A095CA4B6A}</x14:id>
+          <x14:id>{4EF693D8-D0B2-4A99-ABED-A761410E61A0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{893E9808-35B4-4B23-8E3A-9E678260F4AB}</x14:id>
+          <x14:id>{1838A6C1-C2E2-41C8-BBC8-79B177660A5B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{89D2D125-82D9-46BA-AAE0-8A0D7F44A073}">
+          <x14:cfRule type="dataBar" id="{6F640BA9-0B24-4E26-A635-36AF932E75BB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8574E2C1-D780-4071-B61E-C0067B9522CF}">
+          <x14:cfRule type="dataBar" id="{7F9127B5-A116-465D-951E-88D3559AAFE4}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CBBED15E-BBB3-455F-821B-A1A095CA4B6A}">
+          <x14:cfRule type="dataBar" id="{4EF693D8-D0B2-4A99-ABED-A761410E61A0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{893E9808-35B4-4B23-8E3A-9E678260F4AB}">
+          <x14:cfRule type="dataBar" id="{1838A6C1-C2E2-41C8-BBC8-79B177660A5B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: weekly briefing xlsx refresh (universe) 2026-10-23 09:55Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-19.xlsx
+++ b/public/reports/weekly_briefing/2026-10-19.xlsx
@@ -12378,7 +12378,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{07189A70-7105-49DC-AE0D-6C69942BF1D5}</x14:id>
+          <x14:id>{0A13AD2B-F1EA-41CA-858F-ACD02C483824}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12392,7 +12392,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6C72F6D7-DE14-43D2-8115-CC2E4D0ACB7C}</x14:id>
+          <x14:id>{6A9ED66B-70FF-4A99-BE6D-650EB1040484}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12406,7 +12406,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ECDB0782-B748-4AC1-9999-3FCD9B30DB86}</x14:id>
+          <x14:id>{9E87D5F2-74C0-4A22-83F0-600599DC8ED1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12420,7 +12420,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E138A6EC-DEBF-4C7B-A602-99ED8F3A0C8E}</x14:id>
+          <x14:id>{5B870A5A-42D3-4221-A338-4BDE55AE413C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12430,7 +12430,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{07189A70-7105-49DC-AE0D-6C69942BF1D5}">
+          <x14:cfRule type="dataBar" id="{0A13AD2B-F1EA-41CA-858F-ACD02C483824}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12443,7 +12443,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6C72F6D7-DE14-43D2-8115-CC2E4D0ACB7C}">
+          <x14:cfRule type="dataBar" id="{6A9ED66B-70FF-4A99-BE6D-650EB1040484}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12456,7 +12456,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{ECDB0782-B748-4AC1-9999-3FCD9B30DB86}">
+          <x14:cfRule type="dataBar" id="{9E87D5F2-74C0-4A22-83F0-600599DC8ED1}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12469,7 +12469,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E138A6EC-DEBF-4C7B-A602-99ED8F3A0C8E}">
+          <x14:cfRule type="dataBar" id="{5B870A5A-42D3-4221-A338-4BDE55AE413C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27830,7 +27830,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6F640BA9-0B24-4E26-A635-36AF932E75BB}</x14:id>
+          <x14:id>{A5ED43BD-F738-4567-AC28-CF92E470C4DB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27844,7 +27844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7F9127B5-A116-465D-951E-88D3559AAFE4}</x14:id>
+          <x14:id>{67252D63-186F-41EA-868A-470BDBF4B72A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27858,7 +27858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4EF693D8-D0B2-4A99-ABED-A761410E61A0}</x14:id>
+          <x14:id>{D09E8383-0EE5-4D9D-8E39-FEF7CCC205D0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27872,7 +27872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{1838A6C1-C2E2-41C8-BBC8-79B177660A5B}</x14:id>
+          <x14:id>{C0534C05-6CCB-41EF-8688-A7348DC65BBA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -27882,7 +27882,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6F640BA9-0B24-4E26-A635-36AF932E75BB}">
+          <x14:cfRule type="dataBar" id="{A5ED43BD-F738-4567-AC28-CF92E470C4DB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27895,7 +27895,7 @@
           <xm:sqref>N6:N174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7F9127B5-A116-465D-951E-88D3559AAFE4}">
+          <x14:cfRule type="dataBar" id="{67252D63-186F-41EA-868A-470BDBF4B72A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27908,7 +27908,7 @@
           <xm:sqref>P6:P174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4EF693D8-D0B2-4A99-ABED-A761410E61A0}">
+          <x14:cfRule type="dataBar" id="{D09E8383-0EE5-4D9D-8E39-FEF7CCC205D0}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -27921,7 +27921,7 @@
           <xm:sqref>Y6:Y174</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{1838A6C1-C2E2-41C8-BBC8-79B177660A5B}">
+          <x14:cfRule type="dataBar" id="{C0534C05-6CCB-41EF-8688-A7348DC65BBA}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>